<commit_message>
Fix #VALUE! errors in model18 after polish row/column deletes
- Rewrite Scenarios internal column refs when col D is deleted (G→F for base case)
- Rebind Revenue Drivers variance formulas after memo/note row deletes
- Rebind DCF Gordon growth, exit-method, and sensitivity formulas after memo deletes
- Regenerate model18altered.xlsx and model18_final.xlsx

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_final.xlsx
+++ b/LULU/model18_final.xlsx
@@ -1465,7 +1465,7 @@
         </is>
       </c>
       <c r="D10" s="25">
-        <f>E8*E9</f>
+        <f>D8*D9</f>
         <v/>
       </c>
     </row>
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="D13" s="25">
-        <f>E11+E13</f>
+        <f>D11+D13</f>
         <v/>
       </c>
     </row>
@@ -1610,7 +1610,7 @@
         </is>
       </c>
       <c r="D19" s="28">
-        <f>E18/E19</f>
+        <f>D18/D19</f>
         <v/>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
         </is>
       </c>
       <c r="D21" s="28">
-        <f>E17/(1+(1-E5)*E20)</f>
+        <f>D17/(1+(1-D5)*D20)</f>
         <v/>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
         </is>
       </c>
       <c r="D22" s="28">
-        <f>E14/E10</f>
+        <f>D14/D10</f>
         <v/>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
         </is>
       </c>
       <c r="D24" s="29">
-        <f>E22*(1+(1-E5)*E23)</f>
+        <f>D22*(1+(1-D5)*D23)</f>
         <v/>
       </c>
     </row>
@@ -1731,7 +1731,7 @@
         </is>
       </c>
       <c r="D26" s="30">
-        <f>E3+E25*E4</f>
+        <f>D3+D25*D4</f>
         <v/>
       </c>
     </row>
@@ -1770,7 +1770,7 @@
         </is>
       </c>
       <c r="D30" s="31">
-        <f>E35*(1-E5)</f>
+        <f>D35*(1-D5)</f>
         <v/>
       </c>
     </row>
@@ -1799,7 +1799,7 @@
         </is>
       </c>
       <c r="D33" s="32">
-        <f>E10/(E10+E14)</f>
+        <f>D10/(D10+D14)</f>
         <v/>
       </c>
     </row>
@@ -1820,7 +1820,7 @@
         </is>
       </c>
       <c r="D34" s="32">
-        <f>E14/(E10+E14)</f>
+        <f>D14/(D10+D14)</f>
         <v/>
       </c>
     </row>
@@ -1836,7 +1836,7 @@
         </is>
       </c>
       <c r="D35" s="33">
-        <f>E39*E32+E40*E36</f>
+        <f>D39*D32+D40*D36</f>
         <v/>
       </c>
     </row>
@@ -2428,15 +2428,15 @@
         </is>
       </c>
       <c r="E25" s="42">
+        <f>11102600*(1+E4)</f>
+        <v/>
+      </c>
+      <c r="F25" s="42">
         <f>11102600*(1+F4)</f>
         <v/>
       </c>
-      <c r="F25" s="42">
+      <c r="G25" s="42">
         <f>11102600*(1+G4)</f>
-        <v/>
-      </c>
-      <c r="G25" s="42">
-        <f>11102600*(1+H4)</f>
         <v/>
       </c>
     </row>
@@ -2447,15 +2447,15 @@
         </is>
       </c>
       <c r="E26" s="42">
+        <f>E25*(1+E5)</f>
+        <v/>
+      </c>
+      <c r="F26" s="42">
         <f>F25*(1+F5)</f>
         <v/>
       </c>
-      <c r="F26" s="42">
+      <c r="G26" s="42">
         <f>G25*(1+G5)</f>
-        <v/>
-      </c>
-      <c r="G26" s="42">
-        <f>H25*(1+H5)</f>
         <v/>
       </c>
     </row>
@@ -2466,15 +2466,15 @@
         </is>
       </c>
       <c r="E27" s="42">
+        <f>E26*(1+E5)</f>
+        <v/>
+      </c>
+      <c r="F27" s="42">
         <f>F26*(1+F5)</f>
         <v/>
       </c>
-      <c r="F27" s="42">
+      <c r="G27" s="42">
         <f>G26*(1+G5)</f>
-        <v/>
-      </c>
-      <c r="G27" s="42">
-        <f>H26*(1+H5)</f>
         <v/>
       </c>
     </row>
@@ -2485,15 +2485,15 @@
         </is>
       </c>
       <c r="E28" s="42">
+        <f>E27*(1+E5)</f>
+        <v/>
+      </c>
+      <c r="F28" s="42">
         <f>F27*(1+F5)</f>
         <v/>
       </c>
-      <c r="F28" s="42">
+      <c r="G28" s="42">
         <f>G27*(1+G5)</f>
-        <v/>
-      </c>
-      <c r="G28" s="42">
-        <f>H27*(1+H5)</f>
         <v/>
       </c>
     </row>
@@ -2504,15 +2504,15 @@
         </is>
       </c>
       <c r="E29" s="42">
+        <f>E28*(1+E5)</f>
+        <v/>
+      </c>
+      <c r="F29" s="42">
         <f>F28*(1+F5)</f>
         <v/>
       </c>
-      <c r="F29" s="42">
+      <c r="G29" s="42">
         <f>G28*(1+G5)</f>
-        <v/>
-      </c>
-      <c r="G29" s="42">
-        <f>H28*(1+H5)</f>
         <v/>
       </c>
     </row>
@@ -2523,15 +2523,15 @@
         </is>
       </c>
       <c r="E30" s="43">
+        <f>E14</f>
+        <v/>
+      </c>
+      <c r="F30" s="43">
         <f>F14</f>
         <v/>
       </c>
-      <c r="F30" s="43">
+      <c r="G30" s="43">
         <f>G14</f>
-        <v/>
-      </c>
-      <c r="G30" s="43">
-        <f>H14</f>
         <v/>
       </c>
     </row>
@@ -2542,15 +2542,15 @@
         </is>
       </c>
       <c r="E31" s="43">
+        <f>E14</f>
+        <v/>
+      </c>
+      <c r="F31" s="43">
         <f>F14</f>
         <v/>
       </c>
-      <c r="F31" s="43">
+      <c r="G31" s="43">
         <f>G14</f>
-        <v/>
-      </c>
-      <c r="G31" s="43">
-        <f>H14</f>
         <v/>
       </c>
     </row>
@@ -2561,15 +2561,15 @@
         </is>
       </c>
       <c r="E32" s="43">
+        <f>E14</f>
+        <v/>
+      </c>
+      <c r="F32" s="43">
         <f>F14</f>
         <v/>
       </c>
-      <c r="F32" s="43">
+      <c r="G32" s="43">
         <f>G14</f>
-        <v/>
-      </c>
-      <c r="G32" s="43">
-        <f>H14</f>
         <v/>
       </c>
     </row>
@@ -2580,15 +2580,15 @@
         </is>
       </c>
       <c r="E33" s="43">
+        <f>E14</f>
+        <v/>
+      </c>
+      <c r="F33" s="43">
         <f>F14</f>
         <v/>
       </c>
-      <c r="F33" s="43">
+      <c r="G33" s="43">
         <f>G14</f>
-        <v/>
-      </c>
-      <c r="G33" s="43">
-        <f>H14</f>
         <v/>
       </c>
     </row>
@@ -2599,15 +2599,15 @@
         </is>
       </c>
       <c r="E34" s="43">
+        <f>E14</f>
+        <v/>
+      </c>
+      <c r="F34" s="43">
         <f>F14</f>
         <v/>
       </c>
-      <c r="F34" s="43">
+      <c r="G34" s="43">
         <f>G14</f>
-        <v/>
-      </c>
-      <c r="G34" s="43">
-        <f>H14</f>
         <v/>
       </c>
     </row>
@@ -2618,15 +2618,15 @@
         </is>
       </c>
       <c r="E35" s="42">
+        <f>E25*(1-E30)</f>
+        <v/>
+      </c>
+      <c r="F35" s="42">
         <f>F25*(1-F30)</f>
         <v/>
       </c>
-      <c r="F35" s="42">
+      <c r="G35" s="42">
         <f>G25*(1-G30)</f>
-        <v/>
-      </c>
-      <c r="G35" s="42">
-        <f>H25*(1-H30)</f>
         <v/>
       </c>
     </row>
@@ -2637,15 +2637,15 @@
         </is>
       </c>
       <c r="E36" s="42">
+        <f>E26*(1-E31)</f>
+        <v/>
+      </c>
+      <c r="F36" s="42">
         <f>F26*(1-F31)</f>
         <v/>
       </c>
-      <c r="F36" s="42">
+      <c r="G36" s="42">
         <f>G26*(1-G31)</f>
-        <v/>
-      </c>
-      <c r="G36" s="42">
-        <f>H26*(1-H31)</f>
         <v/>
       </c>
     </row>
@@ -2656,15 +2656,15 @@
         </is>
       </c>
       <c r="E37" s="42">
+        <f>E27*(1-E32)</f>
+        <v/>
+      </c>
+      <c r="F37" s="42">
         <f>F27*(1-F32)</f>
         <v/>
       </c>
-      <c r="F37" s="42">
+      <c r="G37" s="42">
         <f>G27*(1-G32)</f>
-        <v/>
-      </c>
-      <c r="G37" s="42">
-        <f>H27*(1-H32)</f>
         <v/>
       </c>
     </row>
@@ -2675,15 +2675,15 @@
         </is>
       </c>
       <c r="E38" s="42">
+        <f>E28*(1-E33)</f>
+        <v/>
+      </c>
+      <c r="F38" s="42">
         <f>F28*(1-F33)</f>
         <v/>
       </c>
-      <c r="F38" s="42">
+      <c r="G38" s="42">
         <f>G28*(1-G33)</f>
-        <v/>
-      </c>
-      <c r="G38" s="42">
-        <f>H28*(1-H33)</f>
         <v/>
       </c>
     </row>
@@ -2694,15 +2694,15 @@
         </is>
       </c>
       <c r="E39" s="42">
+        <f>E29*(1-E34)</f>
+        <v/>
+      </c>
+      <c r="F39" s="42">
         <f>F29*(1-F34)</f>
         <v/>
       </c>
-      <c r="F39" s="42">
+      <c r="G39" s="42">
         <f>G29*(1-G34)</f>
-        <v/>
-      </c>
-      <c r="G39" s="42">
-        <f>H29*(1-H34)</f>
         <v/>
       </c>
     </row>
@@ -2713,15 +2713,15 @@
         </is>
       </c>
       <c r="E40" s="43">
+        <f>E6+(E8-E6)*0/4</f>
+        <v/>
+      </c>
+      <c r="F40" s="43">
         <f>F6+(F8-F6)*0/4</f>
         <v/>
       </c>
-      <c r="F40" s="43">
+      <c r="G40" s="43">
         <f>G6+(G8-G6)*0/4</f>
-        <v/>
-      </c>
-      <c r="G40" s="43">
-        <f>H6+(H8-H6)*0/4</f>
         <v/>
       </c>
     </row>
@@ -2732,15 +2732,15 @@
         </is>
       </c>
       <c r="E41" s="43">
+        <f>E6+(E8-E6)*1/4</f>
+        <v/>
+      </c>
+      <c r="F41" s="43">
         <f>F6+(F8-F6)*1/4</f>
         <v/>
       </c>
-      <c r="F41" s="43">
+      <c r="G41" s="43">
         <f>G6+(G8-G6)*1/4</f>
-        <v/>
-      </c>
-      <c r="G41" s="43">
-        <f>H6+(H8-H6)*1/4</f>
         <v/>
       </c>
     </row>
@@ -2751,15 +2751,15 @@
         </is>
       </c>
       <c r="E42" s="43">
+        <f>E6+(E8-E6)*2/4</f>
+        <v/>
+      </c>
+      <c r="F42" s="43">
         <f>F6+(F8-F6)*2/4</f>
         <v/>
       </c>
-      <c r="F42" s="43">
+      <c r="G42" s="43">
         <f>G6+(G8-G6)*2/4</f>
-        <v/>
-      </c>
-      <c r="G42" s="43">
-        <f>H6+(H8-H6)*2/4</f>
         <v/>
       </c>
     </row>
@@ -2770,15 +2770,15 @@
         </is>
       </c>
       <c r="E43" s="43">
+        <f>E6+(E8-E6)*3/4</f>
+        <v/>
+      </c>
+      <c r="F43" s="43">
         <f>F6+(F8-F6)*3/4</f>
         <v/>
       </c>
-      <c r="F43" s="43">
+      <c r="G43" s="43">
         <f>G6+(G8-G6)*3/4</f>
-        <v/>
-      </c>
-      <c r="G43" s="43">
-        <f>H6+(H8-H6)*3/4</f>
         <v/>
       </c>
     </row>
@@ -2789,15 +2789,15 @@
         </is>
       </c>
       <c r="E44" s="43">
+        <f>E6+(E8-E6)*4/4</f>
+        <v/>
+      </c>
+      <c r="F44" s="43">
         <f>F6+(F8-F6)*4/4</f>
         <v/>
       </c>
-      <c r="F44" s="43">
+      <c r="G44" s="43">
         <f>G6+(G8-G6)*4/4</f>
-        <v/>
-      </c>
-      <c r="G44" s="43">
-        <f>H6+(H8-H6)*4/4</f>
         <v/>
       </c>
     </row>
@@ -2808,15 +2808,15 @@
         </is>
       </c>
       <c r="E45" s="42">
+        <f>E25*E40+E7</f>
+        <v/>
+      </c>
+      <c r="F45" s="42">
         <f>F25*F40+F7</f>
         <v/>
       </c>
-      <c r="F45" s="42">
+      <c r="G45" s="42">
         <f>G25*G40+G7</f>
-        <v/>
-      </c>
-      <c r="G45" s="42">
-        <f>H25*H40+H7</f>
         <v/>
       </c>
     </row>
@@ -2827,15 +2827,15 @@
         </is>
       </c>
       <c r="E46" s="42">
+        <f>E26*E41</f>
+        <v/>
+      </c>
+      <c r="F46" s="42">
         <f>F26*F41</f>
         <v/>
       </c>
-      <c r="F46" s="42">
+      <c r="G46" s="42">
         <f>G26*G41</f>
-        <v/>
-      </c>
-      <c r="G46" s="42">
-        <f>H26*H41</f>
         <v/>
       </c>
     </row>
@@ -2846,15 +2846,15 @@
         </is>
       </c>
       <c r="E47" s="42">
+        <f>E27*E42</f>
+        <v/>
+      </c>
+      <c r="F47" s="42">
         <f>F27*F42</f>
         <v/>
       </c>
-      <c r="F47" s="42">
+      <c r="G47" s="42">
         <f>G27*G42</f>
-        <v/>
-      </c>
-      <c r="G47" s="42">
-        <f>H27*H42</f>
         <v/>
       </c>
     </row>
@@ -2865,15 +2865,15 @@
         </is>
       </c>
       <c r="E48" s="42">
+        <f>E28*E43</f>
+        <v/>
+      </c>
+      <c r="F48" s="42">
         <f>F28*F43</f>
         <v/>
       </c>
-      <c r="F48" s="42">
+      <c r="G48" s="42">
         <f>G28*G43</f>
-        <v/>
-      </c>
-      <c r="G48" s="42">
-        <f>H28*H43</f>
         <v/>
       </c>
     </row>
@@ -2884,15 +2884,15 @@
         </is>
       </c>
       <c r="E49" s="42">
+        <f>E29*E44</f>
+        <v/>
+      </c>
+      <c r="F49" s="42">
         <f>F29*F44</f>
         <v/>
       </c>
-      <c r="F49" s="42">
+      <c r="G49" s="42">
         <f>G29*G44</f>
-        <v/>
-      </c>
-      <c r="G49" s="42">
-        <f>H29*H44</f>
         <v/>
       </c>
     </row>
@@ -2903,7 +2903,7 @@
         </is>
       </c>
       <c r="E50" s="42">
-        <f>F45*(1-'NOPAT Bridge'!E$39)</f>
+        <f>E45*(1-'NOPAT Bridge'!E$39)</f>
         <v/>
       </c>
       <c r="F50" s="42">
@@ -2911,7 +2911,7 @@
         <v/>
       </c>
       <c r="G50" s="42">
-        <f>H45*(1-'NOPAT Bridge'!E$39)</f>
+        <f>G45*(1-'NOPAT Bridge'!E$39)</f>
         <v/>
       </c>
     </row>
@@ -2922,7 +2922,7 @@
         </is>
       </c>
       <c r="E51" s="42">
-        <f>F46*(1-'NOPAT Bridge'!F$39)</f>
+        <f>E46*(1-'NOPAT Bridge'!F$39)</f>
         <v/>
       </c>
       <c r="F51" s="42">
@@ -2930,7 +2930,7 @@
         <v/>
       </c>
       <c r="G51" s="42">
-        <f>H46*(1-'NOPAT Bridge'!F$39)</f>
+        <f>G46*(1-'NOPAT Bridge'!F$39)</f>
         <v/>
       </c>
     </row>
@@ -2941,7 +2941,7 @@
         </is>
       </c>
       <c r="E52" s="42">
-        <f>F47*(1-'NOPAT Bridge'!G$39)</f>
+        <f>E47*(1-'NOPAT Bridge'!G$39)</f>
         <v/>
       </c>
       <c r="F52" s="42">
@@ -2949,7 +2949,7 @@
         <v/>
       </c>
       <c r="G52" s="42">
-        <f>H47*(1-'NOPAT Bridge'!G$39)</f>
+        <f>G47*(1-'NOPAT Bridge'!G$39)</f>
         <v/>
       </c>
     </row>
@@ -2960,7 +2960,7 @@
         </is>
       </c>
       <c r="E53" s="42">
-        <f>F48*(1-'NOPAT Bridge'!H$39)</f>
+        <f>E48*(1-'NOPAT Bridge'!H$39)</f>
         <v/>
       </c>
       <c r="F53" s="42">
@@ -2968,7 +2968,7 @@
         <v/>
       </c>
       <c r="G53" s="42">
-        <f>H48*(1-'NOPAT Bridge'!H$39)</f>
+        <f>G48*(1-'NOPAT Bridge'!H$39)</f>
         <v/>
       </c>
     </row>
@@ -2979,7 +2979,7 @@
         </is>
       </c>
       <c r="E54" s="42">
-        <f>F49*(1-'NOPAT Bridge'!I$39)</f>
+        <f>E49*(1-'NOPAT Bridge'!I$39)</f>
         <v/>
       </c>
       <c r="F54" s="42">
@@ -2987,7 +2987,7 @@
         <v/>
       </c>
       <c r="G54" s="42">
-        <f>H49*(1-'NOPAT Bridge'!I$39)</f>
+        <f>G49*(1-'NOPAT Bridge'!I$39)</f>
         <v/>
       </c>
     </row>
@@ -2998,15 +2998,15 @@
         </is>
       </c>
       <c r="E55" s="42">
+        <f>E25*E12</f>
+        <v/>
+      </c>
+      <c r="F55" s="42">
         <f>F25*F12</f>
         <v/>
       </c>
-      <c r="F55" s="42">
+      <c r="G55" s="42">
         <f>G25*G12</f>
-        <v/>
-      </c>
-      <c r="G55" s="42">
-        <f>H25*H12</f>
         <v/>
       </c>
     </row>
@@ -3017,15 +3017,15 @@
         </is>
       </c>
       <c r="E56" s="42">
+        <f>E26*E12</f>
+        <v/>
+      </c>
+      <c r="F56" s="42">
         <f>F26*F12</f>
         <v/>
       </c>
-      <c r="F56" s="42">
+      <c r="G56" s="42">
         <f>G26*G12</f>
-        <v/>
-      </c>
-      <c r="G56" s="42">
-        <f>H26*H12</f>
         <v/>
       </c>
     </row>
@@ -3036,15 +3036,15 @@
         </is>
       </c>
       <c r="E57" s="42">
+        <f>E27*E12</f>
+        <v/>
+      </c>
+      <c r="F57" s="42">
         <f>F27*F12</f>
         <v/>
       </c>
-      <c r="F57" s="42">
+      <c r="G57" s="42">
         <f>G27*G12</f>
-        <v/>
-      </c>
-      <c r="G57" s="42">
-        <f>H27*H12</f>
         <v/>
       </c>
     </row>
@@ -3055,15 +3055,15 @@
         </is>
       </c>
       <c r="E58" s="42">
+        <f>E28*E12</f>
+        <v/>
+      </c>
+      <c r="F58" s="42">
         <f>F28*F12</f>
         <v/>
       </c>
-      <c r="F58" s="42">
+      <c r="G58" s="42">
         <f>G28*G12</f>
-        <v/>
-      </c>
-      <c r="G58" s="42">
-        <f>H28*H12</f>
         <v/>
       </c>
     </row>
@@ -3074,15 +3074,15 @@
         </is>
       </c>
       <c r="E59" s="42">
+        <f>E29*E12</f>
+        <v/>
+      </c>
+      <c r="F59" s="42">
         <f>F29*F12</f>
         <v/>
       </c>
-      <c r="F59" s="42">
+      <c r="G59" s="42">
         <f>G29*G12</f>
-        <v/>
-      </c>
-      <c r="G59" s="42">
-        <f>H29*H12</f>
         <v/>
       </c>
     </row>
@@ -3093,15 +3093,15 @@
         </is>
       </c>
       <c r="E60" s="42">
+        <f>E25*E13</f>
+        <v/>
+      </c>
+      <c r="F60" s="42">
         <f>F25*F13</f>
         <v/>
       </c>
-      <c r="F60" s="42">
+      <c r="G60" s="42">
         <f>G25*G13</f>
-        <v/>
-      </c>
-      <c r="G60" s="42">
-        <f>H25*H13</f>
         <v/>
       </c>
     </row>
@@ -3112,15 +3112,15 @@
         </is>
       </c>
       <c r="E61" s="42">
+        <f>E26*E13</f>
+        <v/>
+      </c>
+      <c r="F61" s="42">
         <f>F26*F13</f>
         <v/>
       </c>
-      <c r="F61" s="42">
+      <c r="G61" s="42">
         <f>G26*G13</f>
-        <v/>
-      </c>
-      <c r="G61" s="42">
-        <f>H26*H13</f>
         <v/>
       </c>
     </row>
@@ -3131,15 +3131,15 @@
         </is>
       </c>
       <c r="E62" s="42">
+        <f>E27*E13</f>
+        <v/>
+      </c>
+      <c r="F62" s="42">
         <f>F27*F13</f>
         <v/>
       </c>
-      <c r="F62" s="42">
+      <c r="G62" s="42">
         <f>G27*G13</f>
-        <v/>
-      </c>
-      <c r="G62" s="42">
-        <f>H27*H13</f>
         <v/>
       </c>
     </row>
@@ -3150,15 +3150,15 @@
         </is>
       </c>
       <c r="E63" s="42">
+        <f>E28*E13</f>
+        <v/>
+      </c>
+      <c r="F63" s="42">
         <f>F28*F13</f>
         <v/>
       </c>
-      <c r="F63" s="42">
+      <c r="G63" s="42">
         <f>G28*G13</f>
-        <v/>
-      </c>
-      <c r="G63" s="42">
-        <f>H28*H13</f>
         <v/>
       </c>
     </row>
@@ -3169,15 +3169,15 @@
         </is>
       </c>
       <c r="E64" s="42">
+        <f>E29*E13</f>
+        <v/>
+      </c>
+      <c r="F64" s="42">
         <f>F29*F13</f>
         <v/>
       </c>
-      <c r="F64" s="42">
+      <c r="G64" s="42">
         <f>G29*G13</f>
-        <v/>
-      </c>
-      <c r="G64" s="42">
-        <f>H29*H13</f>
         <v/>
       </c>
     </row>
@@ -3188,15 +3188,15 @@
         </is>
       </c>
       <c r="E65" s="44">
+        <f>E15</f>
+        <v/>
+      </c>
+      <c r="F65" s="44">
         <f>F15</f>
         <v/>
       </c>
-      <c r="F65" s="44">
+      <c r="G65" s="44">
         <f>G15</f>
-        <v/>
-      </c>
-      <c r="G65" s="44">
-        <f>H15</f>
         <v/>
       </c>
     </row>
@@ -3207,15 +3207,15 @@
         </is>
       </c>
       <c r="E66" s="44">
+        <f>E15</f>
+        <v/>
+      </c>
+      <c r="F66" s="44">
         <f>F15</f>
         <v/>
       </c>
-      <c r="F66" s="44">
+      <c r="G66" s="44">
         <f>G15</f>
-        <v/>
-      </c>
-      <c r="G66" s="44">
-        <f>H15</f>
         <v/>
       </c>
     </row>
@@ -3226,15 +3226,15 @@
         </is>
       </c>
       <c r="E67" s="44">
+        <f>E15</f>
+        <v/>
+      </c>
+      <c r="F67" s="44">
         <f>F15</f>
         <v/>
       </c>
-      <c r="F67" s="44">
+      <c r="G67" s="44">
         <f>G15</f>
-        <v/>
-      </c>
-      <c r="G67" s="44">
-        <f>H15</f>
         <v/>
       </c>
     </row>
@@ -3245,15 +3245,15 @@
         </is>
       </c>
       <c r="E68" s="44">
+        <f>E15</f>
+        <v/>
+      </c>
+      <c r="F68" s="44">
         <f>F15</f>
         <v/>
       </c>
-      <c r="F68" s="44">
+      <c r="G68" s="44">
         <f>G15</f>
-        <v/>
-      </c>
-      <c r="G68" s="44">
-        <f>H15</f>
         <v/>
       </c>
     </row>
@@ -3264,15 +3264,15 @@
         </is>
       </c>
       <c r="E69" s="44">
+        <f>E15</f>
+        <v/>
+      </c>
+      <c r="F69" s="44">
         <f>F15</f>
         <v/>
       </c>
-      <c r="F69" s="44">
+      <c r="G69" s="44">
         <f>G15</f>
-        <v/>
-      </c>
-      <c r="G69" s="44">
-        <f>H15</f>
         <v/>
       </c>
     </row>
@@ -3283,15 +3283,15 @@
         </is>
       </c>
       <c r="E70" s="42">
+        <f>(E65/365)*E25</f>
+        <v/>
+      </c>
+      <c r="F70" s="42">
         <f>(F65/365)*F25</f>
         <v/>
       </c>
-      <c r="F70" s="42">
+      <c r="G70" s="42">
         <f>(G65/365)*G25</f>
-        <v/>
-      </c>
-      <c r="G70" s="42">
-        <f>(H65/365)*H25</f>
         <v/>
       </c>
     </row>
@@ -3302,15 +3302,15 @@
         </is>
       </c>
       <c r="E71" s="42">
+        <f>(E66/365)*E26</f>
+        <v/>
+      </c>
+      <c r="F71" s="42">
         <f>(F66/365)*F26</f>
         <v/>
       </c>
-      <c r="F71" s="42">
+      <c r="G71" s="42">
         <f>(G66/365)*G26</f>
-        <v/>
-      </c>
-      <c r="G71" s="42">
-        <f>(H66/365)*H26</f>
         <v/>
       </c>
     </row>
@@ -3321,15 +3321,15 @@
         </is>
       </c>
       <c r="E72" s="42">
+        <f>(E67/365)*E27</f>
+        <v/>
+      </c>
+      <c r="F72" s="42">
         <f>(F67/365)*F27</f>
         <v/>
       </c>
-      <c r="F72" s="42">
+      <c r="G72" s="42">
         <f>(G67/365)*G27</f>
-        <v/>
-      </c>
-      <c r="G72" s="42">
-        <f>(H67/365)*H27</f>
         <v/>
       </c>
     </row>
@@ -3340,15 +3340,15 @@
         </is>
       </c>
       <c r="E73" s="42">
+        <f>(E68/365)*E28</f>
+        <v/>
+      </c>
+      <c r="F73" s="42">
         <f>(F68/365)*F28</f>
         <v/>
       </c>
-      <c r="F73" s="42">
+      <c r="G73" s="42">
         <f>(G68/365)*G28</f>
-        <v/>
-      </c>
-      <c r="G73" s="42">
-        <f>(H68/365)*H28</f>
         <v/>
       </c>
     </row>
@@ -3359,15 +3359,15 @@
         </is>
       </c>
       <c r="E74" s="42">
+        <f>(E69/365)*E29</f>
+        <v/>
+      </c>
+      <c r="F74" s="42">
         <f>(F69/365)*F29</f>
         <v/>
       </c>
-      <c r="F74" s="42">
+      <c r="G74" s="42">
         <f>(G69/365)*G29</f>
-        <v/>
-      </c>
-      <c r="G74" s="42">
-        <f>(H69/365)*H29</f>
         <v/>
       </c>
     </row>
@@ -3378,15 +3378,15 @@
         </is>
       </c>
       <c r="E75" s="44">
+        <f>E16-E17*1</f>
+        <v/>
+      </c>
+      <c r="F75" s="44">
         <f>F16-F17*1</f>
         <v/>
       </c>
-      <c r="F75" s="44">
+      <c r="G75" s="44">
         <f>G16-G17*1</f>
-        <v/>
-      </c>
-      <c r="G75" s="44">
-        <f>H16-H17*1</f>
         <v/>
       </c>
     </row>
@@ -3397,15 +3397,15 @@
         </is>
       </c>
       <c r="E76" s="44">
+        <f>E16-E17*2</f>
+        <v/>
+      </c>
+      <c r="F76" s="44">
         <f>F16-F17*2</f>
         <v/>
       </c>
-      <c r="F76" s="44">
+      <c r="G76" s="44">
         <f>G16-G17*2</f>
-        <v/>
-      </c>
-      <c r="G76" s="44">
-        <f>H16-H17*2</f>
         <v/>
       </c>
     </row>
@@ -3416,15 +3416,15 @@
         </is>
       </c>
       <c r="E77" s="44">
+        <f>E16-E17*3</f>
+        <v/>
+      </c>
+      <c r="F77" s="44">
         <f>F16-F17*3</f>
         <v/>
       </c>
-      <c r="F77" s="44">
+      <c r="G77" s="44">
         <f>G16-G17*3</f>
-        <v/>
-      </c>
-      <c r="G77" s="44">
-        <f>H16-H17*3</f>
         <v/>
       </c>
     </row>
@@ -3435,15 +3435,15 @@
         </is>
       </c>
       <c r="E78" s="44">
+        <f>E16-E17*4</f>
+        <v/>
+      </c>
+      <c r="F78" s="44">
         <f>F16-F17*4</f>
         <v/>
       </c>
-      <c r="F78" s="44">
+      <c r="G78" s="44">
         <f>G16-G17*4</f>
-        <v/>
-      </c>
-      <c r="G78" s="44">
-        <f>H16-H17*4</f>
         <v/>
       </c>
     </row>
@@ -3454,15 +3454,15 @@
         </is>
       </c>
       <c r="E79" s="44">
+        <f>E16-E17*5</f>
+        <v/>
+      </c>
+      <c r="F79" s="44">
         <f>F16-F17*5</f>
         <v/>
       </c>
-      <c r="F79" s="44">
+      <c r="G79" s="44">
         <f>G16-G17*5</f>
-        <v/>
-      </c>
-      <c r="G79" s="44">
-        <f>H16-H17*5</f>
         <v/>
       </c>
     </row>
@@ -3473,15 +3473,15 @@
         </is>
       </c>
       <c r="E80" s="42">
+        <f>(E75/365)*E35</f>
+        <v/>
+      </c>
+      <c r="F80" s="42">
         <f>(F75/365)*F35</f>
         <v/>
       </c>
-      <c r="F80" s="42">
+      <c r="G80" s="42">
         <f>(G75/365)*G35</f>
-        <v/>
-      </c>
-      <c r="G80" s="42">
-        <f>(H75/365)*H35</f>
         <v/>
       </c>
     </row>
@@ -3492,15 +3492,15 @@
         </is>
       </c>
       <c r="E81" s="42">
+        <f>(E76/365)*E36</f>
+        <v/>
+      </c>
+      <c r="F81" s="42">
         <f>(F76/365)*F36</f>
         <v/>
       </c>
-      <c r="F81" s="42">
+      <c r="G81" s="42">
         <f>(G76/365)*G36</f>
-        <v/>
-      </c>
-      <c r="G81" s="42">
-        <f>(H76/365)*H36</f>
         <v/>
       </c>
     </row>
@@ -3511,15 +3511,15 @@
         </is>
       </c>
       <c r="E82" s="42">
+        <f>(E77/365)*E37</f>
+        <v/>
+      </c>
+      <c r="F82" s="42">
         <f>(F77/365)*F37</f>
         <v/>
       </c>
-      <c r="F82" s="42">
+      <c r="G82" s="42">
         <f>(G77/365)*G37</f>
-        <v/>
-      </c>
-      <c r="G82" s="42">
-        <f>(H77/365)*H37</f>
         <v/>
       </c>
     </row>
@@ -3530,15 +3530,15 @@
         </is>
       </c>
       <c r="E83" s="42">
+        <f>(E78/365)*E38</f>
+        <v/>
+      </c>
+      <c r="F83" s="42">
         <f>(F78/365)*F38</f>
         <v/>
       </c>
-      <c r="F83" s="42">
+      <c r="G83" s="42">
         <f>(G78/365)*G38</f>
-        <v/>
-      </c>
-      <c r="G83" s="42">
-        <f>(H78/365)*H38</f>
         <v/>
       </c>
     </row>
@@ -3549,15 +3549,15 @@
         </is>
       </c>
       <c r="E84" s="42">
+        <f>(E79/365)*E39</f>
+        <v/>
+      </c>
+      <c r="F84" s="42">
         <f>(F79/365)*F39</f>
         <v/>
       </c>
-      <c r="F84" s="42">
+      <c r="G84" s="42">
         <f>(G79/365)*G39</f>
-        <v/>
-      </c>
-      <c r="G84" s="42">
-        <f>(H79/365)*H39</f>
         <v/>
       </c>
     </row>
@@ -3568,15 +3568,15 @@
         </is>
       </c>
       <c r="E85" s="44">
+        <f>E18</f>
+        <v/>
+      </c>
+      <c r="F85" s="44">
         <f>F18</f>
         <v/>
       </c>
-      <c r="F85" s="44">
+      <c r="G85" s="44">
         <f>G18</f>
-        <v/>
-      </c>
-      <c r="G85" s="44">
-        <f>H18</f>
         <v/>
       </c>
     </row>
@@ -3587,15 +3587,15 @@
         </is>
       </c>
       <c r="E86" s="44">
+        <f>E18</f>
+        <v/>
+      </c>
+      <c r="F86" s="44">
         <f>F18</f>
         <v/>
       </c>
-      <c r="F86" s="44">
+      <c r="G86" s="44">
         <f>G18</f>
-        <v/>
-      </c>
-      <c r="G86" s="44">
-        <f>H18</f>
         <v/>
       </c>
     </row>
@@ -3606,15 +3606,15 @@
         </is>
       </c>
       <c r="E87" s="44">
+        <f>E18</f>
+        <v/>
+      </c>
+      <c r="F87" s="44">
         <f>F18</f>
         <v/>
       </c>
-      <c r="F87" s="44">
+      <c r="G87" s="44">
         <f>G18</f>
-        <v/>
-      </c>
-      <c r="G87" s="44">
-        <f>H18</f>
         <v/>
       </c>
     </row>
@@ -3625,15 +3625,15 @@
         </is>
       </c>
       <c r="E88" s="44">
+        <f>E18</f>
+        <v/>
+      </c>
+      <c r="F88" s="44">
         <f>F18</f>
         <v/>
       </c>
-      <c r="F88" s="44">
+      <c r="G88" s="44">
         <f>G18</f>
-        <v/>
-      </c>
-      <c r="G88" s="44">
-        <f>H18</f>
         <v/>
       </c>
     </row>
@@ -3644,15 +3644,15 @@
         </is>
       </c>
       <c r="E89" s="44">
+        <f>E18</f>
+        <v/>
+      </c>
+      <c r="F89" s="44">
         <f>F18</f>
         <v/>
       </c>
-      <c r="F89" s="44">
+      <c r="G89" s="44">
         <f>G18</f>
-        <v/>
-      </c>
-      <c r="G89" s="44">
-        <f>H18</f>
         <v/>
       </c>
     </row>
@@ -3663,15 +3663,15 @@
         </is>
       </c>
       <c r="E90" s="42">
+        <f>(E85/365)*E35</f>
+        <v/>
+      </c>
+      <c r="F90" s="42">
         <f>(F85/365)*F35</f>
         <v/>
       </c>
-      <c r="F90" s="42">
+      <c r="G90" s="42">
         <f>(G85/365)*G35</f>
-        <v/>
-      </c>
-      <c r="G90" s="42">
-        <f>(H85/365)*H35</f>
         <v/>
       </c>
     </row>
@@ -3682,15 +3682,15 @@
         </is>
       </c>
       <c r="E91" s="42">
+        <f>(E86/365)*E36</f>
+        <v/>
+      </c>
+      <c r="F91" s="42">
         <f>(F86/365)*F36</f>
         <v/>
       </c>
-      <c r="F91" s="42">
+      <c r="G91" s="42">
         <f>(G86/365)*G36</f>
-        <v/>
-      </c>
-      <c r="G91" s="42">
-        <f>(H86/365)*H36</f>
         <v/>
       </c>
     </row>
@@ -3701,15 +3701,15 @@
         </is>
       </c>
       <c r="E92" s="42">
+        <f>(E87/365)*E37</f>
+        <v/>
+      </c>
+      <c r="F92" s="42">
         <f>(F87/365)*F37</f>
         <v/>
       </c>
-      <c r="F92" s="42">
+      <c r="G92" s="42">
         <f>(G87/365)*G37</f>
-        <v/>
-      </c>
-      <c r="G92" s="42">
-        <f>(H87/365)*H37</f>
         <v/>
       </c>
     </row>
@@ -3720,15 +3720,15 @@
         </is>
       </c>
       <c r="E93" s="42">
+        <f>(E88/365)*E38</f>
+        <v/>
+      </c>
+      <c r="F93" s="42">
         <f>(F88/365)*F38</f>
         <v/>
       </c>
-      <c r="F93" s="42">
+      <c r="G93" s="42">
         <f>(G88/365)*G38</f>
-        <v/>
-      </c>
-      <c r="G93" s="42">
-        <f>(H88/365)*H38</f>
         <v/>
       </c>
     </row>
@@ -3739,15 +3739,15 @@
         </is>
       </c>
       <c r="E94" s="42">
+        <f>(E89/365)*E39</f>
+        <v/>
+      </c>
+      <c r="F94" s="42">
         <f>(F89/365)*F39</f>
         <v/>
       </c>
-      <c r="F94" s="42">
+      <c r="G94" s="42">
         <f>(G89/365)*G39</f>
-        <v/>
-      </c>
-      <c r="G94" s="42">
-        <f>(H89/365)*H39</f>
         <v/>
       </c>
     </row>
@@ -3758,15 +3758,15 @@
         </is>
       </c>
       <c r="E95" s="42">
+        <f>E25*E19</f>
+        <v/>
+      </c>
+      <c r="F95" s="42">
         <f>F25*F19</f>
         <v/>
       </c>
-      <c r="F95" s="42">
+      <c r="G95" s="42">
         <f>G25*G19</f>
-        <v/>
-      </c>
-      <c r="G95" s="42">
-        <f>H25*H19</f>
         <v/>
       </c>
     </row>
@@ -3777,15 +3777,15 @@
         </is>
       </c>
       <c r="E96" s="42">
+        <f>E26*E19</f>
+        <v/>
+      </c>
+      <c r="F96" s="42">
         <f>F26*F19</f>
         <v/>
       </c>
-      <c r="F96" s="42">
+      <c r="G96" s="42">
         <f>G26*G19</f>
-        <v/>
-      </c>
-      <c r="G96" s="42">
-        <f>H26*H19</f>
         <v/>
       </c>
     </row>
@@ -3796,15 +3796,15 @@
         </is>
       </c>
       <c r="E97" s="42">
+        <f>E27*E19</f>
+        <v/>
+      </c>
+      <c r="F97" s="42">
         <f>F27*F19</f>
         <v/>
       </c>
-      <c r="F97" s="42">
+      <c r="G97" s="42">
         <f>G27*G19</f>
-        <v/>
-      </c>
-      <c r="G97" s="42">
-        <f>H27*H19</f>
         <v/>
       </c>
     </row>
@@ -3815,15 +3815,15 @@
         </is>
       </c>
       <c r="E98" s="42">
+        <f>E28*E19</f>
+        <v/>
+      </c>
+      <c r="F98" s="42">
         <f>F28*F19</f>
         <v/>
       </c>
-      <c r="F98" s="42">
+      <c r="G98" s="42">
         <f>G28*G19</f>
-        <v/>
-      </c>
-      <c r="G98" s="42">
-        <f>H28*H19</f>
         <v/>
       </c>
     </row>
@@ -3834,15 +3834,15 @@
         </is>
       </c>
       <c r="E99" s="42">
+        <f>E29*E19</f>
+        <v/>
+      </c>
+      <c r="F99" s="42">
         <f>F29*F19</f>
         <v/>
       </c>
-      <c r="F99" s="42">
+      <c r="G99" s="42">
         <f>G29*G19</f>
-        <v/>
-      </c>
-      <c r="G99" s="42">
-        <f>H29*H19</f>
         <v/>
       </c>
     </row>
@@ -3853,15 +3853,15 @@
         </is>
       </c>
       <c r="E100" s="42">
+        <f>E25*E20</f>
+        <v/>
+      </c>
+      <c r="F100" s="42">
         <f>F25*F20</f>
         <v/>
       </c>
-      <c r="F100" s="42">
+      <c r="G100" s="42">
         <f>G25*G20</f>
-        <v/>
-      </c>
-      <c r="G100" s="42">
-        <f>H25*H20</f>
         <v/>
       </c>
     </row>
@@ -3872,15 +3872,15 @@
         </is>
       </c>
       <c r="E101" s="42">
+        <f>E26*E20</f>
+        <v/>
+      </c>
+      <c r="F101" s="42">
         <f>F26*F20</f>
         <v/>
       </c>
-      <c r="F101" s="42">
+      <c r="G101" s="42">
         <f>G26*G20</f>
-        <v/>
-      </c>
-      <c r="G101" s="42">
-        <f>H26*H20</f>
         <v/>
       </c>
     </row>
@@ -3891,15 +3891,15 @@
         </is>
       </c>
       <c r="E102" s="42">
+        <f>E27*E20</f>
+        <v/>
+      </c>
+      <c r="F102" s="42">
         <f>F27*F20</f>
         <v/>
       </c>
-      <c r="F102" s="42">
+      <c r="G102" s="42">
         <f>G27*G20</f>
-        <v/>
-      </c>
-      <c r="G102" s="42">
-        <f>H27*H20</f>
         <v/>
       </c>
     </row>
@@ -3910,15 +3910,15 @@
         </is>
       </c>
       <c r="E103" s="42">
+        <f>E28*E20</f>
+        <v/>
+      </c>
+      <c r="F103" s="42">
         <f>F28*F20</f>
         <v/>
       </c>
-      <c r="F103" s="42">
+      <c r="G103" s="42">
         <f>G28*G20</f>
-        <v/>
-      </c>
-      <c r="G103" s="42">
-        <f>H28*H20</f>
         <v/>
       </c>
     </row>
@@ -3929,15 +3929,15 @@
         </is>
       </c>
       <c r="E104" s="42">
+        <f>E29*E20</f>
+        <v/>
+      </c>
+      <c r="F104" s="42">
         <f>F29*F20</f>
         <v/>
       </c>
-      <c r="F104" s="42">
+      <c r="G104" s="42">
         <f>G29*G20</f>
-        <v/>
-      </c>
-      <c r="G104" s="42">
-        <f>H29*H20</f>
         <v/>
       </c>
     </row>
@@ -3948,15 +3948,15 @@
         </is>
       </c>
       <c r="E105" s="42">
+        <f>E70+E80+E95</f>
+        <v/>
+      </c>
+      <c r="F105" s="42">
         <f>F70+F80+F95</f>
         <v/>
       </c>
-      <c r="F105" s="42">
+      <c r="G105" s="42">
         <f>G70+G80+G95</f>
-        <v/>
-      </c>
-      <c r="G105" s="42">
-        <f>H70+H80+H95</f>
         <v/>
       </c>
     </row>
@@ -3967,15 +3967,15 @@
         </is>
       </c>
       <c r="E106" s="42">
+        <f>E71+E81+E96</f>
+        <v/>
+      </c>
+      <c r="F106" s="42">
         <f>F71+F81+F96</f>
         <v/>
       </c>
-      <c r="F106" s="42">
+      <c r="G106" s="42">
         <f>G71+G81+G96</f>
-        <v/>
-      </c>
-      <c r="G106" s="42">
-        <f>H71+H81+H96</f>
         <v/>
       </c>
     </row>
@@ -3986,15 +3986,15 @@
         </is>
       </c>
       <c r="E107" s="42">
+        <f>E72+E82+E97</f>
+        <v/>
+      </c>
+      <c r="F107" s="42">
         <f>F72+F82+F97</f>
         <v/>
       </c>
-      <c r="F107" s="42">
+      <c r="G107" s="42">
         <f>G72+G82+G97</f>
-        <v/>
-      </c>
-      <c r="G107" s="42">
-        <f>H72+H82+H97</f>
         <v/>
       </c>
     </row>
@@ -4005,15 +4005,15 @@
         </is>
       </c>
       <c r="E108" s="42">
+        <f>E73+E83+E98</f>
+        <v/>
+      </c>
+      <c r="F108" s="42">
         <f>F73+F83+F98</f>
         <v/>
       </c>
-      <c r="F108" s="42">
+      <c r="G108" s="42">
         <f>G73+G83+G98</f>
-        <v/>
-      </c>
-      <c r="G108" s="42">
-        <f>H73+H83+H98</f>
         <v/>
       </c>
     </row>
@@ -4024,15 +4024,15 @@
         </is>
       </c>
       <c r="E109" s="42">
+        <f>E74+E84+E99</f>
+        <v/>
+      </c>
+      <c r="F109" s="42">
         <f>F74+F84+F99</f>
         <v/>
       </c>
-      <c r="F109" s="42">
+      <c r="G109" s="42">
         <f>G74+G84+G99</f>
-        <v/>
-      </c>
-      <c r="G109" s="42">
-        <f>H74+H84+H99</f>
         <v/>
       </c>
     </row>
@@ -4043,15 +4043,15 @@
         </is>
       </c>
       <c r="E110" s="42">
+        <f>E90+E100</f>
+        <v/>
+      </c>
+      <c r="F110" s="42">
         <f>F90+F100</f>
         <v/>
       </c>
-      <c r="F110" s="42">
+      <c r="G110" s="42">
         <f>G90+G100</f>
-        <v/>
-      </c>
-      <c r="G110" s="42">
-        <f>H90+H100</f>
         <v/>
       </c>
     </row>
@@ -4062,15 +4062,15 @@
         </is>
       </c>
       <c r="E111" s="42">
+        <f>E91+E101</f>
+        <v/>
+      </c>
+      <c r="F111" s="42">
         <f>F91+F101</f>
         <v/>
       </c>
-      <c r="F111" s="42">
+      <c r="G111" s="42">
         <f>G91+G101</f>
-        <v/>
-      </c>
-      <c r="G111" s="42">
-        <f>H91+H101</f>
         <v/>
       </c>
     </row>
@@ -4081,15 +4081,15 @@
         </is>
       </c>
       <c r="E112" s="42">
+        <f>E92+E102</f>
+        <v/>
+      </c>
+      <c r="F112" s="42">
         <f>F92+F102</f>
         <v/>
       </c>
-      <c r="F112" s="42">
+      <c r="G112" s="42">
         <f>G92+G102</f>
-        <v/>
-      </c>
-      <c r="G112" s="42">
-        <f>H92+H102</f>
         <v/>
       </c>
     </row>
@@ -4100,15 +4100,15 @@
         </is>
       </c>
       <c r="E113" s="42">
+        <f>E93+E103</f>
+        <v/>
+      </c>
+      <c r="F113" s="42">
         <f>F93+F103</f>
         <v/>
       </c>
-      <c r="F113" s="42">
+      <c r="G113" s="42">
         <f>G93+G103</f>
-        <v/>
-      </c>
-      <c r="G113" s="42">
-        <f>H93+H103</f>
         <v/>
       </c>
     </row>
@@ -4119,15 +4119,15 @@
         </is>
       </c>
       <c r="E114" s="42">
+        <f>E94+E104</f>
+        <v/>
+      </c>
+      <c r="F114" s="42">
         <f>F94+F104</f>
         <v/>
       </c>
-      <c r="F114" s="42">
+      <c r="G114" s="42">
         <f>G94+G104</f>
-        <v/>
-      </c>
-      <c r="G114" s="42">
-        <f>H94+H104</f>
         <v/>
       </c>
     </row>
@@ -4138,15 +4138,15 @@
         </is>
       </c>
       <c r="E115" s="42">
+        <f>E105-E110</f>
+        <v/>
+      </c>
+      <c r="F115" s="42">
         <f>F105-F110</f>
         <v/>
       </c>
-      <c r="F115" s="42">
+      <c r="G115" s="42">
         <f>G105-G110</f>
-        <v/>
-      </c>
-      <c r="G115" s="42">
-        <f>H105-H110</f>
         <v/>
       </c>
     </row>
@@ -4157,15 +4157,15 @@
         </is>
       </c>
       <c r="E116" s="42">
+        <f>E106-E111</f>
+        <v/>
+      </c>
+      <c r="F116" s="42">
         <f>F106-F111</f>
         <v/>
       </c>
-      <c r="F116" s="42">
+      <c r="G116" s="42">
         <f>G106-G111</f>
-        <v/>
-      </c>
-      <c r="G116" s="42">
-        <f>H106-H111</f>
         <v/>
       </c>
     </row>
@@ -4176,15 +4176,15 @@
         </is>
       </c>
       <c r="E117" s="42">
+        <f>E107-E112</f>
+        <v/>
+      </c>
+      <c r="F117" s="42">
         <f>F107-F112</f>
         <v/>
       </c>
-      <c r="F117" s="42">
+      <c r="G117" s="42">
         <f>G107-G112</f>
-        <v/>
-      </c>
-      <c r="G117" s="42">
-        <f>H107-H112</f>
         <v/>
       </c>
     </row>
@@ -4195,15 +4195,15 @@
         </is>
       </c>
       <c r="E118" s="42">
+        <f>E108-E113</f>
+        <v/>
+      </c>
+      <c r="F118" s="42">
         <f>F108-F113</f>
         <v/>
       </c>
-      <c r="F118" s="42">
+      <c r="G118" s="42">
         <f>G108-G113</f>
-        <v/>
-      </c>
-      <c r="G118" s="42">
-        <f>H108-H113</f>
         <v/>
       </c>
     </row>
@@ -4214,15 +4214,15 @@
         </is>
       </c>
       <c r="E119" s="42">
+        <f>E109-E114</f>
+        <v/>
+      </c>
+      <c r="F119" s="42">
         <f>F109-F114</f>
         <v/>
       </c>
-      <c r="F119" s="42">
+      <c r="G119" s="42">
         <f>G109-G114</f>
-        <v/>
-      </c>
-      <c r="G119" s="42">
-        <f>H109-H114</f>
         <v/>
       </c>
     </row>
@@ -4233,15 +4233,15 @@
         </is>
       </c>
       <c r="E120" s="42">
+        <f>1461096-E115</f>
+        <v/>
+      </c>
+      <c r="F120" s="42">
         <f>1461096-F115</f>
         <v/>
       </c>
-      <c r="F120" s="42">
+      <c r="G120" s="42">
         <f>1461096-G115</f>
-        <v/>
-      </c>
-      <c r="G120" s="42">
-        <f>1461096-H115</f>
         <v/>
       </c>
     </row>
@@ -4252,15 +4252,15 @@
         </is>
       </c>
       <c r="E121" s="42">
+        <f>E115-E116</f>
+        <v/>
+      </c>
+      <c r="F121" s="42">
         <f>F115-F116</f>
         <v/>
       </c>
-      <c r="F121" s="42">
+      <c r="G121" s="42">
         <f>G115-G116</f>
-        <v/>
-      </c>
-      <c r="G121" s="42">
-        <f>H115-H116</f>
         <v/>
       </c>
     </row>
@@ -4271,15 +4271,15 @@
         </is>
       </c>
       <c r="E122" s="42">
+        <f>E116-E117</f>
+        <v/>
+      </c>
+      <c r="F122" s="42">
         <f>F116-F117</f>
         <v/>
       </c>
-      <c r="F122" s="42">
+      <c r="G122" s="42">
         <f>G116-G117</f>
-        <v/>
-      </c>
-      <c r="G122" s="42">
-        <f>H116-H117</f>
         <v/>
       </c>
     </row>
@@ -4290,15 +4290,15 @@
         </is>
       </c>
       <c r="E123" s="42">
+        <f>E117-E118</f>
+        <v/>
+      </c>
+      <c r="F123" s="42">
         <f>F117-F118</f>
         <v/>
       </c>
-      <c r="F123" s="42">
+      <c r="G123" s="42">
         <f>G117-G118</f>
-        <v/>
-      </c>
-      <c r="G123" s="42">
-        <f>H117-H118</f>
         <v/>
       </c>
     </row>
@@ -4309,15 +4309,15 @@
         </is>
       </c>
       <c r="E124" s="42">
+        <f>E118-E119</f>
+        <v/>
+      </c>
+      <c r="F124" s="42">
         <f>F118-F119</f>
         <v/>
       </c>
-      <c r="F124" s="42">
+      <c r="G124" s="42">
         <f>G118-G119</f>
-        <v/>
-      </c>
-      <c r="G124" s="42">
-        <f>H118-H119</f>
         <v/>
       </c>
     </row>
@@ -4328,15 +4328,15 @@
         </is>
       </c>
       <c r="E125" s="42">
+        <f>E50+E55-E60+E120</f>
+        <v/>
+      </c>
+      <c r="F125" s="42">
         <f>F50+F55-F60+F120</f>
         <v/>
       </c>
-      <c r="F125" s="42">
+      <c r="G125" s="42">
         <f>G50+G55-G60+G120</f>
-        <v/>
-      </c>
-      <c r="G125" s="42">
-        <f>H50+H55-H60+H120</f>
         <v/>
       </c>
     </row>
@@ -4347,15 +4347,15 @@
         </is>
       </c>
       <c r="E126" s="42">
+        <f>E51+E56-E61+E121</f>
+        <v/>
+      </c>
+      <c r="F126" s="42">
         <f>F51+F56-F61+F121</f>
         <v/>
       </c>
-      <c r="F126" s="42">
+      <c r="G126" s="42">
         <f>G51+G56-G61+G121</f>
-        <v/>
-      </c>
-      <c r="G126" s="42">
-        <f>H51+H56-H61+H121</f>
         <v/>
       </c>
     </row>
@@ -4366,15 +4366,15 @@
         </is>
       </c>
       <c r="E127" s="42">
+        <f>E52+E57-E62+E122</f>
+        <v/>
+      </c>
+      <c r="F127" s="42">
         <f>F52+F57-F62+F122</f>
         <v/>
       </c>
-      <c r="F127" s="42">
+      <c r="G127" s="42">
         <f>G52+G57-G62+G122</f>
-        <v/>
-      </c>
-      <c r="G127" s="42">
-        <f>H52+H57-H62+H122</f>
         <v/>
       </c>
     </row>
@@ -4385,15 +4385,15 @@
         </is>
       </c>
       <c r="E128" s="42">
+        <f>E53+E58-E63+E123</f>
+        <v/>
+      </c>
+      <c r="F128" s="42">
         <f>F53+F58-F63+F123</f>
         <v/>
       </c>
-      <c r="F128" s="42">
+      <c r="G128" s="42">
         <f>G53+G58-G63+G123</f>
-        <v/>
-      </c>
-      <c r="G128" s="42">
-        <f>H53+H58-H63+H123</f>
         <v/>
       </c>
     </row>
@@ -4404,15 +4404,15 @@
         </is>
       </c>
       <c r="E129" s="42">
+        <f>E54+E59-E64+E124</f>
+        <v/>
+      </c>
+      <c r="F129" s="42">
         <f>F54+F59-F64+F124</f>
         <v/>
       </c>
-      <c r="F129" s="42">
+      <c r="G129" s="42">
         <f>G54+G59-G64+G124</f>
-        <v/>
-      </c>
-      <c r="G129" s="42">
-        <f>H54+H59-H64+H124</f>
         <v/>
       </c>
     </row>
@@ -4424,15 +4424,15 @@
         </is>
       </c>
       <c r="E131" s="25">
+        <f>NPV(E9,E125,E126,E127,E128,E129)+(E129*(1+E10)/(E9-E10))/(1+E9)^5</f>
+        <v/>
+      </c>
+      <c r="F131" s="25">
         <f>NPV(F9,F125,F126,F127,F128,F129)+(F129*(1+F10)/(F9-F10))/(1+F9)^5</f>
         <v/>
       </c>
-      <c r="F131" s="25">
+      <c r="G131" s="25">
         <f>NPV(G9,G125,G126,G127,G128,G129)+(G129*(1+G10)/(G9-G10))/(1+G9)^5</f>
-        <v/>
-      </c>
-      <c r="G131" s="25">
-        <f>NPV(H9,H125,H126,H127,H128,H129)+(H129*(1+H10)/(H9-H10))/(1+H9)^5</f>
         <v/>
       </c>
     </row>
@@ -4443,15 +4443,15 @@
         </is>
       </c>
       <c r="E132" s="46">
+        <f>(E131+1807202-1798441)/111380</f>
+        <v/>
+      </c>
+      <c r="F132" s="47">
         <f>(F131+1807202-1798441)/111380</f>
         <v/>
       </c>
-      <c r="F132" s="47">
+      <c r="G132" s="46">
         <f>(G131+1807202-1798441)/111380</f>
-        <v/>
-      </c>
-      <c r="G132" s="46">
-        <f>(H131+1807202-1798441)/111380</f>
         <v/>
       </c>
     </row>
@@ -4462,15 +4462,15 @@
         </is>
       </c>
       <c r="E133" s="48">
+        <f>E132/100.0-1</f>
+        <v/>
+      </c>
+      <c r="F133" s="48">
         <f>F132/100.0-1</f>
         <v/>
       </c>
-      <c r="F133" s="48">
+      <c r="G133" s="48">
         <f>G132/100.0-1</f>
-        <v/>
-      </c>
-      <c r="G133" s="48">
-        <f>H132/100.0-1</f>
         <v/>
       </c>
     </row>
@@ -4577,15 +4577,15 @@
         </is>
       </c>
       <c r="E143" s="42">
+        <f>(E45+E138)*(1-E11)</f>
+        <v/>
+      </c>
+      <c r="F143" s="42">
         <f>(F45+F138)*(1-F11)</f>
         <v/>
       </c>
-      <c r="F143" s="42">
+      <c r="G143" s="42">
         <f>(G45+G138)*(1-G11)</f>
-        <v/>
-      </c>
-      <c r="G143" s="42">
-        <f>(H45+H138)*(1-H11)</f>
         <v/>
       </c>
     </row>
@@ -4596,15 +4596,15 @@
         </is>
       </c>
       <c r="E144" s="42">
+        <f>(E46+E139)*(1-E11)</f>
+        <v/>
+      </c>
+      <c r="F144" s="42">
         <f>(F46+F139)*(1-F11)</f>
         <v/>
       </c>
-      <c r="F144" s="42">
+      <c r="G144" s="42">
         <f>(G46+G139)*(1-G11)</f>
-        <v/>
-      </c>
-      <c r="G144" s="42">
-        <f>(H46+H139)*(1-H11)</f>
         <v/>
       </c>
     </row>
@@ -4615,15 +4615,15 @@
         </is>
       </c>
       <c r="E145" s="42">
+        <f>(E47+E140)*(1-E11)</f>
+        <v/>
+      </c>
+      <c r="F145" s="42">
         <f>(F47+F140)*(1-F11)</f>
         <v/>
       </c>
-      <c r="F145" s="42">
+      <c r="G145" s="42">
         <f>(G47+G140)*(1-G11)</f>
-        <v/>
-      </c>
-      <c r="G145" s="42">
-        <f>(H47+H140)*(1-H11)</f>
         <v/>
       </c>
     </row>
@@ -4634,15 +4634,15 @@
         </is>
       </c>
       <c r="E146" s="42">
+        <f>(E48+E141)*(1-E11)</f>
+        <v/>
+      </c>
+      <c r="F146" s="42">
         <f>(F48+F141)*(1-F11)</f>
         <v/>
       </c>
-      <c r="F146" s="42">
+      <c r="G146" s="42">
         <f>(G48+G141)*(1-G11)</f>
-        <v/>
-      </c>
-      <c r="G146" s="42">
-        <f>(H48+H141)*(1-H11)</f>
         <v/>
       </c>
     </row>
@@ -4653,15 +4653,15 @@
         </is>
       </c>
       <c r="E147" s="42">
+        <f>(E49+E142)*(1-E11)</f>
+        <v/>
+      </c>
+      <c r="F147" s="42">
         <f>(F49+F142)*(1-F11)</f>
         <v/>
       </c>
-      <c r="F147" s="42">
+      <c r="G147" s="42">
         <f>(G49+G142)*(1-G11)</f>
-        <v/>
-      </c>
-      <c r="G147" s="42">
-        <f>(H49+H142)*(1-H11)</f>
         <v/>
       </c>
     </row>
@@ -4672,15 +4672,15 @@
         </is>
       </c>
       <c r="E148" s="42">
+        <f>E143+E55+E120</f>
+        <v/>
+      </c>
+      <c r="F148" s="42">
         <f>F143+F55+F120</f>
         <v/>
       </c>
-      <c r="F148" s="42">
+      <c r="G148" s="42">
         <f>G143+G55+G120</f>
-        <v/>
-      </c>
-      <c r="G148" s="42">
-        <f>H143+H55+H120</f>
         <v/>
       </c>
     </row>
@@ -4691,15 +4691,15 @@
         </is>
       </c>
       <c r="E149" s="42">
+        <f>E144+E56+E121</f>
+        <v/>
+      </c>
+      <c r="F149" s="42">
         <f>F144+F56+F121</f>
         <v/>
       </c>
-      <c r="F149" s="42">
+      <c r="G149" s="42">
         <f>G144+G56+G121</f>
-        <v/>
-      </c>
-      <c r="G149" s="42">
-        <f>H144+H56+H121</f>
         <v/>
       </c>
     </row>
@@ -4710,15 +4710,15 @@
         </is>
       </c>
       <c r="E150" s="42">
+        <f>E145+E57+E122</f>
+        <v/>
+      </c>
+      <c r="F150" s="42">
         <f>F145+F57+F122</f>
         <v/>
       </c>
-      <c r="F150" s="42">
+      <c r="G150" s="42">
         <f>G145+G57+G122</f>
-        <v/>
-      </c>
-      <c r="G150" s="42">
-        <f>H145+H57+H122</f>
         <v/>
       </c>
     </row>
@@ -4729,15 +4729,15 @@
         </is>
       </c>
       <c r="E151" s="42">
+        <f>E146+E58+E123</f>
+        <v/>
+      </c>
+      <c r="F151" s="42">
         <f>F146+F58+F123</f>
         <v/>
       </c>
-      <c r="F151" s="42">
+      <c r="G151" s="42">
         <f>G146+G58+G123</f>
-        <v/>
-      </c>
-      <c r="G151" s="42">
-        <f>H146+H58+H123</f>
         <v/>
       </c>
     </row>
@@ -4748,15 +4748,15 @@
         </is>
       </c>
       <c r="E152" s="42">
+        <f>E147+E59+E124</f>
+        <v/>
+      </c>
+      <c r="F152" s="42">
         <f>F147+F59+F124</f>
         <v/>
       </c>
-      <c r="F152" s="42">
+      <c r="G152" s="42">
         <f>G147+G59+G124</f>
-        <v/>
-      </c>
-      <c r="G152" s="42">
-        <f>H147+H59+H124</f>
         <v/>
       </c>
     </row>
@@ -4767,15 +4767,15 @@
         </is>
       </c>
       <c r="E153" s="42">
+        <f>E148-E60</f>
+        <v/>
+      </c>
+      <c r="F153" s="42">
         <f>F148-F60</f>
         <v/>
       </c>
-      <c r="F153" s="42">
+      <c r="G153" s="42">
         <f>G148-G60</f>
-        <v/>
-      </c>
-      <c r="G153" s="42">
-        <f>H148-H60</f>
         <v/>
       </c>
     </row>
@@ -4786,15 +4786,15 @@
         </is>
       </c>
       <c r="E154" s="42">
+        <f>E149-E61</f>
+        <v/>
+      </c>
+      <c r="F154" s="42">
         <f>F149-F61</f>
         <v/>
       </c>
-      <c r="F154" s="42">
+      <c r="G154" s="42">
         <f>G149-G61</f>
-        <v/>
-      </c>
-      <c r="G154" s="42">
-        <f>H149-H61</f>
         <v/>
       </c>
     </row>
@@ -4805,15 +4805,15 @@
         </is>
       </c>
       <c r="E155" s="42">
+        <f>E150-E62</f>
+        <v/>
+      </c>
+      <c r="F155" s="42">
         <f>F150-F62</f>
         <v/>
       </c>
-      <c r="F155" s="42">
+      <c r="G155" s="42">
         <f>G150-G62</f>
-        <v/>
-      </c>
-      <c r="G155" s="42">
-        <f>H150-H62</f>
         <v/>
       </c>
     </row>
@@ -4824,15 +4824,15 @@
         </is>
       </c>
       <c r="E156" s="42">
+        <f>E151-E63</f>
+        <v/>
+      </c>
+      <c r="F156" s="42">
         <f>F151-F63</f>
         <v/>
       </c>
-      <c r="F156" s="42">
+      <c r="G156" s="42">
         <f>G151-G63</f>
-        <v/>
-      </c>
-      <c r="G156" s="42">
-        <f>H151-H63</f>
         <v/>
       </c>
     </row>
@@ -4843,15 +4843,15 @@
         </is>
       </c>
       <c r="E157" s="42">
+        <f>E152-E64</f>
+        <v/>
+      </c>
+      <c r="F157" s="42">
         <f>F152-F64</f>
         <v/>
       </c>
-      <c r="F157" s="42">
+      <c r="G157" s="42">
         <f>G152-G64</f>
-        <v/>
-      </c>
-      <c r="G157" s="42">
-        <f>H152-H64</f>
         <v/>
       </c>
     </row>
@@ -4862,15 +4862,15 @@
         </is>
       </c>
       <c r="E158" s="42">
+        <f>-E21</f>
+        <v/>
+      </c>
+      <c r="F158" s="42">
         <f>-F21</f>
         <v/>
       </c>
-      <c r="F158" s="42">
-        <f>-G21</f>
-        <v/>
-      </c>
       <c r="G158" s="42">
-        <f>-ROUND(H22*H153,0)</f>
+        <f>-ROUND(G22*G153,0)</f>
         <v/>
       </c>
     </row>
@@ -4881,15 +4881,15 @@
         </is>
       </c>
       <c r="E159" s="42">
+        <f>-E21</f>
+        <v/>
+      </c>
+      <c r="F159" s="42">
         <f>-F21</f>
         <v/>
       </c>
-      <c r="F159" s="42">
-        <f>-G21</f>
-        <v/>
-      </c>
       <c r="G159" s="42">
-        <f>-ROUND(H22*H154,0)</f>
+        <f>-ROUND(G22*G154,0)</f>
         <v/>
       </c>
     </row>
@@ -4900,15 +4900,15 @@
         </is>
       </c>
       <c r="E160" s="42">
+        <f>-E21</f>
+        <v/>
+      </c>
+      <c r="F160" s="42">
         <f>-F21</f>
         <v/>
       </c>
-      <c r="F160" s="42">
-        <f>-G21</f>
-        <v/>
-      </c>
       <c r="G160" s="42">
-        <f>-ROUND(H22*H155,0)</f>
+        <f>-ROUND(G22*G155,0)</f>
         <v/>
       </c>
     </row>
@@ -4919,15 +4919,15 @@
         </is>
       </c>
       <c r="E161" s="42">
+        <f>-E21</f>
+        <v/>
+      </c>
+      <c r="F161" s="42">
         <f>-F21</f>
         <v/>
       </c>
-      <c r="F161" s="42">
-        <f>-G21</f>
-        <v/>
-      </c>
       <c r="G161" s="42">
-        <f>-ROUND(H22*H156,0)</f>
+        <f>-ROUND(G22*G156,0)</f>
         <v/>
       </c>
     </row>
@@ -4938,15 +4938,15 @@
         </is>
       </c>
       <c r="E162" s="42">
+        <f>-E21</f>
+        <v/>
+      </c>
+      <c r="F162" s="42">
         <f>-F21</f>
         <v/>
       </c>
-      <c r="F162" s="42">
-        <f>-G21</f>
-        <v/>
-      </c>
       <c r="G162" s="42">
-        <f>-ROUND(H22*H157,0)</f>
+        <f>-ROUND(G22*G157,0)</f>
         <v/>
       </c>
     </row>
@@ -4957,15 +4957,15 @@
         </is>
       </c>
       <c r="E163" s="42">
+        <f>1807202+E153+E158</f>
+        <v/>
+      </c>
+      <c r="F163" s="42">
         <f>1807202+F153+F158</f>
         <v/>
       </c>
-      <c r="F163" s="42">
+      <c r="G163" s="42">
         <f>1807202+G153+G158</f>
-        <v/>
-      </c>
-      <c r="G163" s="42">
-        <f>1807202+H153+H158</f>
         <v/>
       </c>
     </row>
@@ -4976,15 +4976,15 @@
         </is>
       </c>
       <c r="E164" s="42">
+        <f>E163+E154+E159</f>
+        <v/>
+      </c>
+      <c r="F164" s="42">
         <f>F163+F154+F159</f>
         <v/>
       </c>
-      <c r="F164" s="42">
+      <c r="G164" s="42">
         <f>G163+G154+G159</f>
-        <v/>
-      </c>
-      <c r="G164" s="42">
-        <f>H163+H154+H159</f>
         <v/>
       </c>
     </row>
@@ -4995,15 +4995,15 @@
         </is>
       </c>
       <c r="E165" s="42">
+        <f>E164+E155+E160</f>
+        <v/>
+      </c>
+      <c r="F165" s="42">
         <f>F164+F155+F160</f>
         <v/>
       </c>
-      <c r="F165" s="42">
+      <c r="G165" s="42">
         <f>G164+G155+G160</f>
-        <v/>
-      </c>
-      <c r="G165" s="42">
-        <f>H164+H155+H160</f>
         <v/>
       </c>
     </row>
@@ -5014,15 +5014,15 @@
         </is>
       </c>
       <c r="E166" s="42">
+        <f>E165+E156+E161</f>
+        <v/>
+      </c>
+      <c r="F166" s="42">
         <f>F165+F156+F161</f>
         <v/>
       </c>
-      <c r="F166" s="42">
+      <c r="G166" s="42">
         <f>G165+G156+G161</f>
-        <v/>
-      </c>
-      <c r="G166" s="42">
-        <f>H165+H156+H161</f>
         <v/>
       </c>
     </row>
@@ -5033,15 +5033,15 @@
         </is>
       </c>
       <c r="E167" s="42">
+        <f>E166+E157+E162</f>
+        <v/>
+      </c>
+      <c r="F167" s="42">
         <f>F166+F157+F162</f>
         <v/>
       </c>
-      <c r="F167" s="42">
+      <c r="G167" s="42">
         <f>G166+G157+G162</f>
-        <v/>
-      </c>
-      <c r="G167" s="42">
-        <f>H166+H157+H162</f>
         <v/>
       </c>
     </row>
@@ -5052,15 +5052,15 @@
         </is>
       </c>
       <c r="E168" s="42">
+        <f>8456743*E25/11102600</f>
+        <v/>
+      </c>
+      <c r="F168" s="42">
         <f>8456743*F25/11102600</f>
         <v/>
       </c>
-      <c r="F168" s="42">
+      <c r="G168" s="42">
         <f>8456743*G25/11102600</f>
-        <v/>
-      </c>
-      <c r="G168" s="42">
-        <f>8456743*H25/11102600</f>
         <v/>
       </c>
     </row>
@@ -5071,15 +5071,15 @@
         </is>
       </c>
       <c r="E169" s="42">
+        <f>8456743*E26/11102600</f>
+        <v/>
+      </c>
+      <c r="F169" s="42">
         <f>8456743*F26/11102600</f>
         <v/>
       </c>
-      <c r="F169" s="42">
+      <c r="G169" s="42">
         <f>8456743*G26/11102600</f>
-        <v/>
-      </c>
-      <c r="G169" s="42">
-        <f>8456743*H26/11102600</f>
         <v/>
       </c>
     </row>
@@ -5090,15 +5090,15 @@
         </is>
       </c>
       <c r="E170" s="42">
+        <f>8456743*E27/11102600</f>
+        <v/>
+      </c>
+      <c r="F170" s="42">
         <f>8456743*F27/11102600</f>
         <v/>
       </c>
-      <c r="F170" s="42">
+      <c r="G170" s="42">
         <f>8456743*G27/11102600</f>
-        <v/>
-      </c>
-      <c r="G170" s="42">
-        <f>8456743*H27/11102600</f>
         <v/>
       </c>
     </row>
@@ -5109,15 +5109,15 @@
         </is>
       </c>
       <c r="E171" s="42">
+        <f>8456743*E28/11102600</f>
+        <v/>
+      </c>
+      <c r="F171" s="42">
         <f>8456743*F28/11102600</f>
         <v/>
       </c>
-      <c r="F171" s="42">
+      <c r="G171" s="42">
         <f>8456743*G28/11102600</f>
-        <v/>
-      </c>
-      <c r="G171" s="42">
-        <f>8456743*H28/11102600</f>
         <v/>
       </c>
     </row>
@@ -5128,15 +5128,15 @@
         </is>
       </c>
       <c r="E172" s="42">
+        <f>8456743*E29/11102600</f>
+        <v/>
+      </c>
+      <c r="F172" s="42">
         <f>8456743*F29/11102600</f>
         <v/>
       </c>
-      <c r="F172" s="42">
+      <c r="G172" s="42">
         <f>8456743*G29/11102600</f>
-        <v/>
-      </c>
-      <c r="G172" s="42">
-        <f>8456743*H29/11102600</f>
         <v/>
       </c>
     </row>
@@ -5147,15 +5147,15 @@
         </is>
       </c>
       <c r="E173" s="42">
+        <f>3494903*E25/11102600</f>
+        <v/>
+      </c>
+      <c r="F173" s="42">
         <f>3494903*F25/11102600</f>
         <v/>
       </c>
-      <c r="F173" s="42">
+      <c r="G173" s="42">
         <f>3494903*G25/11102600</f>
-        <v/>
-      </c>
-      <c r="G173" s="42">
-        <f>3494903*H25/11102600</f>
         <v/>
       </c>
     </row>
@@ -5166,15 +5166,15 @@
         </is>
       </c>
       <c r="E174" s="42">
+        <f>3494903*E26/11102600</f>
+        <v/>
+      </c>
+      <c r="F174" s="42">
         <f>3494903*F26/11102600</f>
         <v/>
       </c>
-      <c r="F174" s="42">
+      <c r="G174" s="42">
         <f>3494903*G26/11102600</f>
-        <v/>
-      </c>
-      <c r="G174" s="42">
-        <f>3494903*H26/11102600</f>
         <v/>
       </c>
     </row>
@@ -5185,15 +5185,15 @@
         </is>
       </c>
       <c r="E175" s="42">
+        <f>3494903*E27/11102600</f>
+        <v/>
+      </c>
+      <c r="F175" s="42">
         <f>3494903*F27/11102600</f>
         <v/>
       </c>
-      <c r="F175" s="42">
+      <c r="G175" s="42">
         <f>3494903*G27/11102600</f>
-        <v/>
-      </c>
-      <c r="G175" s="42">
-        <f>3494903*H27/11102600</f>
         <v/>
       </c>
     </row>
@@ -5204,15 +5204,15 @@
         </is>
       </c>
       <c r="E176" s="42">
+        <f>3494903*E28/11102600</f>
+        <v/>
+      </c>
+      <c r="F176" s="42">
         <f>3494903*F28/11102600</f>
         <v/>
       </c>
-      <c r="F176" s="42">
+      <c r="G176" s="42">
         <f>3494903*G28/11102600</f>
-        <v/>
-      </c>
-      <c r="G176" s="42">
-        <f>3494903*H28/11102600</f>
         <v/>
       </c>
     </row>
@@ -5223,15 +5223,15 @@
         </is>
       </c>
       <c r="E177" s="42">
+        <f>3494903*E29/11102600</f>
+        <v/>
+      </c>
+      <c r="F177" s="42">
         <f>3494903*F29/11102600</f>
         <v/>
       </c>
-      <c r="F177" s="42">
+      <c r="G177" s="42">
         <f>3494903*G29/11102600</f>
-        <v/>
-      </c>
-      <c r="G177" s="42">
-        <f>3494903*H29/11102600</f>
         <v/>
       </c>
     </row>
@@ -5242,15 +5242,15 @@
         </is>
       </c>
       <c r="E178" s="42">
+        <f>4961840*E25/11102600</f>
+        <v/>
+      </c>
+      <c r="F178" s="42">
         <f>4961840*F25/11102600</f>
         <v/>
       </c>
-      <c r="F178" s="42">
+      <c r="G178" s="42">
         <f>4961840*G25/11102600</f>
-        <v/>
-      </c>
-      <c r="G178" s="42">
-        <f>4961840*H25/11102600</f>
         <v/>
       </c>
     </row>
@@ -5261,15 +5261,15 @@
         </is>
       </c>
       <c r="E179" s="42">
+        <f>4961840*E26/11102600</f>
+        <v/>
+      </c>
+      <c r="F179" s="42">
         <f>4961840*F26/11102600</f>
         <v/>
       </c>
-      <c r="F179" s="42">
+      <c r="G179" s="42">
         <f>4961840*G26/11102600</f>
-        <v/>
-      </c>
-      <c r="G179" s="42">
-        <f>4961840*H26/11102600</f>
         <v/>
       </c>
     </row>
@@ -5280,15 +5280,15 @@
         </is>
       </c>
       <c r="E180" s="42">
+        <f>4961840*E27/11102600</f>
+        <v/>
+      </c>
+      <c r="F180" s="42">
         <f>4961840*F27/11102600</f>
         <v/>
       </c>
-      <c r="F180" s="42">
+      <c r="G180" s="42">
         <f>4961840*G27/11102600</f>
-        <v/>
-      </c>
-      <c r="G180" s="42">
-        <f>4961840*H27/11102600</f>
         <v/>
       </c>
     </row>
@@ -5299,15 +5299,15 @@
         </is>
       </c>
       <c r="E181" s="42">
+        <f>4961840*E28/11102600</f>
+        <v/>
+      </c>
+      <c r="F181" s="42">
         <f>4961840*F28/11102600</f>
         <v/>
       </c>
-      <c r="F181" s="42">
+      <c r="G181" s="42">
         <f>4961840*G28/11102600</f>
-        <v/>
-      </c>
-      <c r="G181" s="42">
-        <f>4961840*H28/11102600</f>
         <v/>
       </c>
     </row>
@@ -5318,15 +5318,15 @@
         </is>
       </c>
       <c r="E182" s="42">
+        <f>4961840*E29/11102600</f>
+        <v/>
+      </c>
+      <c r="F182" s="42">
         <f>4961840*F29/11102600</f>
         <v/>
       </c>
-      <c r="F182" s="42">
+      <c r="G182" s="42">
         <f>4961840*G29/11102600</f>
-        <v/>
-      </c>
-      <c r="G182" s="42">
-        <f>4961840*H29/11102600</f>
         <v/>
       </c>
     </row>
@@ -5337,15 +5337,15 @@
         </is>
       </c>
       <c r="E183" s="42">
+        <f>119068-E21/100</f>
+        <v/>
+      </c>
+      <c r="F183" s="42">
         <f>119068-F21/100</f>
         <v/>
       </c>
-      <c r="F183" s="42">
-        <f>119068-G21/100</f>
-        <v/>
-      </c>
       <c r="G183" s="42">
-        <f>119068-ROUND(H22*H153,0)/100</f>
+        <f>119068-ROUND(G22*G153,0)/100</f>
         <v/>
       </c>
     </row>
@@ -5356,15 +5356,15 @@
         </is>
       </c>
       <c r="E184" s="42">
+        <f>E183-E21/108</f>
+        <v/>
+      </c>
+      <c r="F184" s="42">
         <f>F183-F21/108</f>
         <v/>
       </c>
-      <c r="F184" s="42">
-        <f>G183-G21/108</f>
-        <v/>
-      </c>
       <c r="G184" s="42">
-        <f>H183-ROUND(H22*H154,0)/108</f>
+        <f>G183-ROUND(G22*G154,0)/108</f>
         <v/>
       </c>
     </row>
@@ -5375,15 +5375,15 @@
         </is>
       </c>
       <c r="E185" s="42">
+        <f>E184-E21/115</f>
+        <v/>
+      </c>
+      <c r="F185" s="42">
         <f>F184-F21/115</f>
         <v/>
       </c>
-      <c r="F185" s="42">
-        <f>G184-G21/115</f>
-        <v/>
-      </c>
       <c r="G185" s="42">
-        <f>H184-ROUND(H22*H155,0)/115</f>
+        <f>G184-ROUND(G22*G155,0)/115</f>
         <v/>
       </c>
     </row>
@@ -5394,15 +5394,15 @@
         </is>
       </c>
       <c r="E186" s="42">
+        <f>E185-E21/122</f>
+        <v/>
+      </c>
+      <c r="F186" s="42">
         <f>F185-F21/122</f>
         <v/>
       </c>
-      <c r="F186" s="42">
-        <f>G185-G21/122</f>
-        <v/>
-      </c>
       <c r="G186" s="42">
-        <f>H185-ROUND(H22*H156,0)/122</f>
+        <f>G185-ROUND(G22*G156,0)/122</f>
         <v/>
       </c>
     </row>
@@ -5413,15 +5413,15 @@
         </is>
       </c>
       <c r="E187" s="42">
+        <f>E186-E21/130</f>
+        <v/>
+      </c>
+      <c r="F187" s="42">
         <f>F186-F21/130</f>
         <v/>
       </c>
-      <c r="F187" s="42">
-        <f>G186-G21/130</f>
-        <v/>
-      </c>
       <c r="G187" s="42">
-        <f>H186-ROUND(H22*H157,0)/130</f>
+        <f>G186-ROUND(G22*G157,0)/130</f>
         <v/>
       </c>
     </row>
@@ -5432,15 +5432,15 @@
         </is>
       </c>
       <c r="E188" s="49">
+        <f>E143/E183</f>
+        <v/>
+      </c>
+      <c r="F188" s="49">
         <f>F143/F183</f>
         <v/>
       </c>
-      <c r="F188" s="49">
+      <c r="G188" s="49">
         <f>G143/G183</f>
-        <v/>
-      </c>
-      <c r="G188" s="49">
-        <f>H143/H183</f>
         <v/>
       </c>
     </row>
@@ -5451,15 +5451,15 @@
         </is>
       </c>
       <c r="E189" s="49">
+        <f>E144/E184</f>
+        <v/>
+      </c>
+      <c r="F189" s="49">
         <f>F144/F184</f>
         <v/>
       </c>
-      <c r="F189" s="49">
+      <c r="G189" s="49">
         <f>G144/G184</f>
-        <v/>
-      </c>
-      <c r="G189" s="49">
-        <f>H144/H184</f>
         <v/>
       </c>
     </row>
@@ -5470,15 +5470,15 @@
         </is>
       </c>
       <c r="E190" s="49">
+        <f>E145/E185</f>
+        <v/>
+      </c>
+      <c r="F190" s="49">
         <f>F145/F185</f>
         <v/>
       </c>
-      <c r="F190" s="49">
+      <c r="G190" s="49">
         <f>G145/G185</f>
-        <v/>
-      </c>
-      <c r="G190" s="49">
-        <f>H145/H185</f>
         <v/>
       </c>
     </row>
@@ -5489,15 +5489,15 @@
         </is>
       </c>
       <c r="E191" s="49">
+        <f>E146/E186</f>
+        <v/>
+      </c>
+      <c r="F191" s="49">
         <f>F146/F186</f>
         <v/>
       </c>
-      <c r="F191" s="49">
+      <c r="G191" s="49">
         <f>G146/G186</f>
-        <v/>
-      </c>
-      <c r="G191" s="49">
-        <f>H146/H186</f>
         <v/>
       </c>
     </row>
@@ -5508,15 +5508,15 @@
         </is>
       </c>
       <c r="E192" s="49">
+        <f>E147/E187</f>
+        <v/>
+      </c>
+      <c r="F192" s="49">
         <f>F147/F187</f>
         <v/>
       </c>
-      <c r="F192" s="49">
+      <c r="G192" s="49">
         <f>G147/G187</f>
-        <v/>
-      </c>
-      <c r="G192" s="49">
-        <f>H147/H187</f>
         <v/>
       </c>
     </row>
@@ -7246,27 +7246,27 @@
         </is>
       </c>
       <c r="B54" s="42">
-        <f>B55-B56</f>
+        <f>B52-B53</f>
         <v/>
       </c>
       <c r="C54" s="42">
-        <f>C55-C56</f>
+        <f>C52-C53</f>
         <v/>
       </c>
       <c r="D54" s="42">
-        <f>D55-D56</f>
+        <f>D52-D53</f>
         <v/>
       </c>
       <c r="E54" s="42">
-        <f>E55-E56</f>
+        <f>E52-E53</f>
         <v/>
       </c>
       <c r="F54" s="42">
-        <f>F55-F56</f>
+        <f>F52-F53</f>
         <v/>
       </c>
       <c r="G54" s="42">
-        <f>G55-G56</f>
+        <f>G52-G53</f>
         <v/>
       </c>
       <c r="I54" s="17" t="inlineStr">
@@ -7282,27 +7282,27 @@
         </is>
       </c>
       <c r="B55" s="43">
-        <f>IF(B56=0,"",B57/B56)</f>
+        <f>IF(B53=0,"",B54/B53)</f>
         <v/>
       </c>
       <c r="C55" s="43">
-        <f>IF(C56=0,"",C57/C56)</f>
+        <f>IF(C53=0,"",C54/C53)</f>
         <v/>
       </c>
       <c r="D55" s="43">
-        <f>IF(D56=0,"",D57/D56)</f>
+        <f>IF(D53=0,"",D54/D53)</f>
         <v/>
       </c>
       <c r="E55" s="43">
-        <f>IF(E56=0,"",E57/E56)</f>
+        <f>IF(E53=0,"",E54/E53)</f>
         <v/>
       </c>
       <c r="F55" s="43">
-        <f>IF(F56=0,"",F57/F56)</f>
+        <f>IF(F53=0,"",F54/F53)</f>
         <v/>
       </c>
       <c r="G55" s="43">
-        <f>IF(G56=0,"",G57/G56)</f>
+        <f>IF(G53=0,"",G54/G53)</f>
         <v/>
       </c>
       <c r="I55" s="17" t="inlineStr">
@@ -7824,27 +7824,27 @@
         </is>
       </c>
       <c r="D20" s="75">
-        <f>62203*$E$7</f>
+        <f>62203*$D$7</f>
         <v/>
       </c>
       <c r="E20" s="75">
-        <f>Scenarios!F25/11102600*62203*$E$7</f>
+        <f>Scenarios!F25/11102600*62203*$D$7</f>
         <v/>
       </c>
       <c r="F20" s="75">
-        <f>Scenarios!F26/11102600*62203*$E$7</f>
+        <f>Scenarios!F26/11102600*62203*$D$7</f>
         <v/>
       </c>
       <c r="G20" s="75">
-        <f>Scenarios!F27/11102600*62203*$E$7</f>
+        <f>Scenarios!F27/11102600*62203*$D$7</f>
         <v/>
       </c>
       <c r="H20" s="75">
-        <f>Scenarios!F28/11102600*62203*$E$7</f>
+        <f>Scenarios!F28/11102600*62203*$D$7</f>
         <v/>
       </c>
       <c r="I20" s="75">
-        <f>Scenarios!F29/11102600*62203*$E$7</f>
+        <f>Scenarios!F29/11102600*62203*$D$7</f>
         <v/>
       </c>
     </row>
@@ -7864,23 +7864,23 @@
         </is>
       </c>
       <c r="E21" s="25">
+        <f>E16+E17+E18+E19+E20</f>
+        <v/>
+      </c>
+      <c r="F21" s="25">
         <f>F16+F17+F18+F19+F20</f>
         <v/>
       </c>
-      <c r="F21" s="25">
+      <c r="G21" s="25">
         <f>G16+G17+G18+G19+G20</f>
         <v/>
       </c>
-      <c r="G21" s="25">
+      <c r="H21" s="25">
         <f>H16+H17+H18+H19+H20</f>
         <v/>
       </c>
-      <c r="H21" s="25">
+      <c r="I21" s="25">
         <f>I16+I17+I18+I19+I20</f>
-        <v/>
-      </c>
-      <c r="I21" s="25">
-        <f>J16+J17+J18+J19+J20</f>
         <v/>
       </c>
     </row>
@@ -8017,23 +8017,23 @@
         </is>
       </c>
       <c r="E26" s="25">
+        <f>E21+E23+E24-E25</f>
+        <v/>
+      </c>
+      <c r="F26" s="25">
         <f>F21+F23+F24-F25</f>
         <v/>
       </c>
-      <c r="F26" s="25">
+      <c r="G26" s="25">
         <f>G21+G23+G24-G25</f>
         <v/>
       </c>
-      <c r="G26" s="25">
+      <c r="H26" s="25">
         <f>H21+H23+H24-H25</f>
         <v/>
       </c>
-      <c r="H26" s="25">
+      <c r="I26" s="25">
         <f>I21+I23+I24-I25</f>
-        <v/>
-      </c>
-      <c r="I26" s="25">
-        <f>J21+J23+J24-J25</f>
         <v/>
       </c>
     </row>
@@ -8181,27 +8181,27 @@
         </is>
       </c>
       <c r="D31" s="126">
-        <f>E28*$E$9</f>
+        <f>D28*$D$9</f>
         <v/>
       </c>
       <c r="E31" s="75">
-        <f>F28*E$9</f>
+        <f>E28*D$9</f>
         <v/>
       </c>
       <c r="F31" s="75">
-        <f>G28*E$9</f>
+        <f>F28*D$9</f>
         <v/>
       </c>
       <c r="G31" s="75">
-        <f>H28*E$9</f>
+        <f>G28*D$9</f>
         <v/>
       </c>
       <c r="H31" s="75">
-        <f>I28*E$9</f>
+        <f>H28*D$9</f>
         <v/>
       </c>
       <c r="I31" s="75">
-        <f>J28*E$9</f>
+        <f>I28*D$9</f>
         <v/>
       </c>
     </row>
@@ -8222,27 +8222,27 @@
         </is>
       </c>
       <c r="D32" s="126">
-        <f>E29*$E$10</f>
+        <f>D29*$D$10</f>
         <v/>
       </c>
       <c r="E32" s="75">
-        <f>F29*E$10</f>
+        <f>E29*D$10</f>
         <v/>
       </c>
       <c r="F32" s="75">
-        <f>G29*E$10</f>
+        <f>F29*D$10</f>
         <v/>
       </c>
       <c r="G32" s="75">
-        <f>H29*E$10</f>
+        <f>G29*D$10</f>
         <v/>
       </c>
       <c r="H32" s="75">
-        <f>I29*E$10</f>
+        <f>H29*D$10</f>
         <v/>
       </c>
       <c r="I32" s="75">
-        <f>J29*E$10</f>
+        <f>I29*D$10</f>
         <v/>
       </c>
     </row>
@@ -8263,27 +8263,27 @@
         </is>
       </c>
       <c r="D33" s="126">
-        <f>E30*$E$11</f>
+        <f>D30*$D$11</f>
         <v/>
       </c>
       <c r="E33" s="75">
-        <f>F30*E$11</f>
+        <f>E30*D$11</f>
         <v/>
       </c>
       <c r="F33" s="75">
-        <f>G30*E$11</f>
+        <f>F30*D$11</f>
         <v/>
       </c>
       <c r="G33" s="75">
-        <f>H30*E$11</f>
+        <f>G30*D$11</f>
         <v/>
       </c>
       <c r="H33" s="75">
-        <f>I30*E$11</f>
+        <f>H30*D$11</f>
         <v/>
       </c>
       <c r="I33" s="75">
-        <f>J30*E$11</f>
+        <f>I30*D$11</f>
         <v/>
       </c>
     </row>
@@ -8304,23 +8304,23 @@
         </is>
       </c>
       <c r="E34" s="70">
-        <f>F31+F32+F33+Scenarios!F7</f>
+        <f>E31+E32+E33+Scenarios!F7</f>
         <v/>
       </c>
       <c r="F34" s="70">
+        <f>F31+F32+F33</f>
+        <v/>
+      </c>
+      <c r="G34" s="70">
         <f>G31+G32+G33</f>
         <v/>
       </c>
-      <c r="G34" s="70">
+      <c r="H34" s="70">
         <f>H31+H32+H33</f>
         <v/>
       </c>
-      <c r="H34" s="70">
+      <c r="I34" s="70">
         <f>I31+I32+I33</f>
-        <v/>
-      </c>
-      <c r="I34" s="70">
-        <f>J31+J32+J33</f>
         <v/>
       </c>
     </row>
@@ -8340,27 +8340,27 @@
         </is>
       </c>
       <c r="D35" s="127">
-        <f>E31+E32+E33</f>
+        <f>D31+D32+D33</f>
         <v/>
       </c>
       <c r="E35" s="25">
+        <f>E34</f>
+        <v/>
+      </c>
+      <c r="F35" s="25">
         <f>F34</f>
         <v/>
       </c>
-      <c r="F35" s="25">
+      <c r="G35" s="25">
         <f>G34</f>
         <v/>
       </c>
-      <c r="G35" s="25">
+      <c r="H35" s="25">
         <f>H34</f>
         <v/>
       </c>
-      <c r="H35" s="25">
+      <c r="I35" s="25">
         <f>I34</f>
-        <v/>
-      </c>
-      <c r="I35" s="25">
-        <f>J34</f>
         <v/>
       </c>
     </row>
@@ -8380,7 +8380,7 @@
         </is>
       </c>
       <c r="D36" s="25">
-        <f>E21+E23+E24-E25</f>
+        <f>D21+D23+D24-D25</f>
         <v/>
       </c>
       <c r="E36" s="25">
@@ -8411,23 +8411,23 @@
         </is>
       </c>
       <c r="E37" s="75">
-        <f>F36-Scenarios!F45</f>
+        <f>E36-Scenarios!F45</f>
         <v/>
       </c>
       <c r="F37" s="75">
-        <f>G36-Scenarios!F46</f>
+        <f>F36-Scenarios!F46</f>
         <v/>
       </c>
       <c r="G37" s="75">
-        <f>H36-Scenarios!F47</f>
+        <f>G36-Scenarios!F47</f>
         <v/>
       </c>
       <c r="H37" s="75">
-        <f>I36-Scenarios!F48</f>
+        <f>H36-Scenarios!F48</f>
         <v/>
       </c>
       <c r="I37" s="75">
-        <f>J36-Scenarios!F49</f>
+        <f>I36-Scenarios!F49</f>
         <v/>
       </c>
     </row>
@@ -8459,23 +8459,23 @@
         <v/>
       </c>
       <c r="E39" s="32">
-        <f>0.29468476492135026+(F$12-0.29468476492135026)*1/5</f>
+        <f>0.29468476492135026+(E$12-0.29468476492135026)*1/5</f>
         <v/>
       </c>
       <c r="F39" s="32">
-        <f>0.29468476492135026+(G$12-0.29468476492135026)*2/5</f>
+        <f>0.29468476492135026+(F$12-0.29468476492135026)*2/5</f>
         <v/>
       </c>
       <c r="G39" s="32">
-        <f>0.29468476492135026+(H$12-0.29468476492135026)*3/5</f>
+        <f>0.29468476492135026+(G$12-0.29468476492135026)*3/5</f>
         <v/>
       </c>
       <c r="H39" s="32">
-        <f>0.29468476492135026+(I$12-0.29468476492135026)*4/5</f>
+        <f>0.29468476492135026+(H$12-0.29468476492135026)*4/5</f>
         <v/>
       </c>
       <c r="I39" s="32">
-        <f>0.29468476492135026+(J$12-0.29468476492135026)*5/5</f>
+        <f>0.29468476492135026+(I$12-0.29468476492135026)*5/5</f>
         <v/>
       </c>
     </row>
@@ -8496,23 +8496,23 @@
         </is>
       </c>
       <c r="E40" s="75">
+        <f>E36*E39</f>
+        <v/>
+      </c>
+      <c r="F40" s="75">
         <f>F36*F39</f>
         <v/>
       </c>
-      <c r="F40" s="75">
+      <c r="G40" s="75">
         <f>G36*G39</f>
         <v/>
       </c>
-      <c r="G40" s="75">
+      <c r="H40" s="75">
         <f>H36*H39</f>
         <v/>
       </c>
-      <c r="H40" s="75">
+      <c r="I40" s="75">
         <f>I36*I39</f>
-        <v/>
-      </c>
-      <c r="I40" s="75">
-        <f>J36*J39</f>
         <v/>
       </c>
     </row>
@@ -8533,23 +8533,23 @@
         </is>
       </c>
       <c r="E41" s="25">
+        <f>E36-E40</f>
+        <v/>
+      </c>
+      <c r="F41" s="25">
         <f>F36-F40</f>
         <v/>
       </c>
-      <c r="F41" s="25">
+      <c r="G41" s="25">
         <f>G36-G40</f>
         <v/>
       </c>
-      <c r="G41" s="25">
+      <c r="H41" s="25">
         <f>H36-H40</f>
         <v/>
       </c>
-      <c r="H41" s="25">
+      <c r="I41" s="25">
         <f>I36-I40</f>
-        <v/>
-      </c>
-      <c r="I41" s="25">
-        <f>J36-J40</f>
         <v/>
       </c>
     </row>
@@ -9947,7 +9947,7 @@
         </is>
       </c>
       <c r="E45" s="94">
-        <f>E45/E44</f>
+        <f>E44/E43</f>
         <v/>
       </c>
     </row>
@@ -9958,7 +9958,7 @@
         </is>
       </c>
       <c r="E46" s="70">
-        <f>E45/(1+Scenarios!$F$9)^J36</f>
+        <f>E44/(1+Scenarios!$F$9)^J36</f>
         <v/>
       </c>
     </row>
@@ -9969,7 +9969,7 @@
         </is>
       </c>
       <c r="E47" s="25">
-        <f>E42+E48</f>
+        <f>E41+E46</f>
         <v/>
       </c>
     </row>
@@ -10018,7 +10018,7 @@
         </is>
       </c>
       <c r="E50" s="25">
-        <f>E49+E50+E51</f>
+        <f>E47+E48+E49</f>
         <v/>
       </c>
     </row>
@@ -10045,7 +10045,7 @@
         </is>
       </c>
       <c r="E52" s="96">
-        <f>E54/E55</f>
+        <f>E50/E51</f>
         <v/>
       </c>
       <c r="K52" s="87">
@@ -10076,7 +10076,7 @@
         </is>
       </c>
       <c r="E54" s="98">
-        <f>E56/E57-1</f>
+        <f>E52/E53-1</f>
         <v/>
       </c>
     </row>
@@ -10114,7 +10114,7 @@
     <row r="58">
       <c r="A58" s="26" t="inlineStr">
         <is>
-          <t>Guardrail: implied value per share above still divides equity value by Day-1 shares (E55 = 111,380k). This schedule does not change intrinsic DCF per share.</t>
+          <t>Guardrail: implied value per share above still divides equity value by Day-1 shares (E51 = 111,380k). This schedule does not change intrinsic DCF per share.</t>
         </is>
       </c>
     </row>
@@ -10484,7 +10484,7 @@
         </is>
       </c>
       <c r="E78" s="75">
-        <f>E44*E82</f>
+        <f>E43*E77</f>
         <v/>
       </c>
     </row>
@@ -10495,7 +10495,7 @@
         </is>
       </c>
       <c r="E79" s="75">
-        <f>E83/(1+Scenarios!$F$9)^J36</f>
+        <f>E78/(1+Scenarios!$F$9)^J36</f>
         <v/>
       </c>
     </row>
@@ -10506,7 +10506,7 @@
         </is>
       </c>
       <c r="E80" s="25">
-        <f>E42+E84</f>
+        <f>E41+E79</f>
         <v/>
       </c>
     </row>
@@ -10517,7 +10517,7 @@
         </is>
       </c>
       <c r="E81" s="102">
-        <f>(E85+E50+E51)/E55</f>
+        <f>(E80+E48+E49)/E51</f>
         <v/>
       </c>
     </row>
@@ -10674,23 +10674,23 @@
       </c>
       <c r="D94" s="19" t="n"/>
       <c r="F94" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E50+E51)/E55</f>
+        <f>(NPV(0.095,F35:J35)+(J35*(1+0.015)/(0.095-0.015))/(1+0.095)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="G94" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E50+E51)/E55</f>
+        <f>(NPV(0.095,F35:J35)+(J35*(1+0.02)/(0.095-0.02))/(1+0.095)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="H94" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E50+E51)/E55</f>
+        <f>(NPV(0.095,F35:J35)+(J35*(1+0.0225)/(0.095-0.0225))/(1+0.095)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="I94" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E50+E51)/E55</f>
+        <f>(NPV(0.095,F35:J35)+(J35*(1+0.025)/(0.095-0.025))/(1+0.095)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="J94" s="110">
-        <f>(NPV(0.095,F35:J35)+(J35*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E50+E51)/E55</f>
+        <f>(NPV(0.095,F35:J35)+(J35*(1+0.03)/(0.095-0.03))/(1+0.095)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="L94" s="95" t="inlineStr">
@@ -10705,23 +10705,23 @@
       </c>
       <c r="D95" s="19" t="n"/>
       <c r="F95" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E50+E51)/E55</f>
+        <f>(NPV(0.1,F35:J35)+(J35*(1+0.015)/(0.1-0.015))/(1+0.1)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="G95" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E50+E51)/E55</f>
+        <f>(NPV(0.1,F35:J35)+(J35*(1+0.02)/(0.1-0.02))/(1+0.1)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="H95" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E50+E51)/E55</f>
+        <f>(NPV(0.1,F35:J35)+(J35*(1+0.0225)/(0.1-0.0225))/(1+0.1)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="I95" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E50+E51)/E55</f>
+        <f>(NPV(0.1,F35:J35)+(J35*(1+0.025)/(0.1-0.025))/(1+0.1)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="J95" s="110">
-        <f>(NPV(0.1,F35:J35)+(J35*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E50+E51)/E55</f>
+        <f>(NPV(0.1,F35:J35)+(J35*(1+0.03)/(0.1-0.03))/(1+0.1)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="L95" s="95" t="inlineStr">
@@ -10736,23 +10736,23 @@
       </c>
       <c r="D96" s="19" t="n"/>
       <c r="F96" s="110">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E50+E51)/E55</f>
+        <f>(NPV(0.105,F35:J35)+(J35*(1+0.015)/(0.105-0.015))/(1+0.105)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="G96" s="110">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E50+E51)/E55</f>
+        <f>(NPV(0.105,F35:J35)+(J35*(1+0.02)/(0.105-0.02))/(1+0.105)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="H96" s="111">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E50+E51)/E55</f>
+        <f>(NPV(0.105,F35:J35)+(J35*(1+0.0225)/(0.105-0.0225))/(1+0.105)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="I96" s="110">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E50+E51)/E55</f>
+        <f>(NPV(0.105,F35:J35)+(J35*(1+0.025)/(0.105-0.025))/(1+0.105)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="J96" s="110">
-        <f>(NPV(0.105,F35:J35)+(J35*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E50+E51)/E55</f>
+        <f>(NPV(0.105,F35:J35)+(J35*(1+0.03)/(0.105-0.03))/(1+0.105)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="L96" s="95" t="inlineStr">
@@ -10767,23 +10767,23 @@
       </c>
       <c r="D97" s="19" t="n"/>
       <c r="F97" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E50+E51)/E55</f>
+        <f>(NPV(0.11,F35:J35)+(J35*(1+0.015)/(0.11-0.015))/(1+0.11)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="G97" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E50+E51)/E55</f>
+        <f>(NPV(0.11,F35:J35)+(J35*(1+0.02)/(0.11-0.02))/(1+0.11)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="H97" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E50+E51)/E55</f>
+        <f>(NPV(0.11,F35:J35)+(J35*(1+0.0225)/(0.11-0.0225))/(1+0.11)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="I97" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E50+E51)/E55</f>
+        <f>(NPV(0.11,F35:J35)+(J35*(1+0.025)/(0.11-0.025))/(1+0.11)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="J97" s="110">
-        <f>(NPV(0.11,F35:J35)+(J35*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E50+E51)/E55</f>
+        <f>(NPV(0.11,F35:J35)+(J35*(1+0.03)/(0.11-0.03))/(1+0.11)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="L97" s="95" t="inlineStr">
@@ -10803,23 +10803,23 @@
       </c>
       <c r="D98" s="19" t="n"/>
       <c r="F98" s="110">
-        <f>(NPV(0.115,F35:J35)+(J35*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E50+E51)/E55</f>
+        <f>(NPV(0.115,F35:J35)+(J35*(1+0.015)/(0.115-0.015))/(1+0.115)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="G98" s="110">
-        <f>(NPV(0.115,F35:J35)+(J35*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E50+E51)/E55</f>
+        <f>(NPV(0.115,F35:J35)+(J35*(1+0.02)/(0.115-0.02))/(1+0.115)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="H98" s="110">
-        <f>(NPV(0.115,F35:J35)+(J35*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E50+E51)/E55</f>
+        <f>(NPV(0.115,F35:J35)+(J35*(1+0.0225)/(0.115-0.0225))/(1+0.115)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="I98" s="110">
-        <f>(NPV(0.115,F35:J35)+(J35*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E50+E51)/E55</f>
+        <f>(NPV(0.115,F35:J35)+(J35*(1+0.025)/(0.115-0.025))/(1+0.115)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="J98" s="110">
-        <f>(NPV(0.115,F35:J35)+(J35*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E50+E51)/E55</f>
+        <f>(NPV(0.115,F35:J35)+(J35*(1+0.03)/(0.115-0.03))/(1+0.115)^5+E48+E49)/E51</f>
         <v/>
       </c>
       <c r="L98" s="95" t="inlineStr">
@@ -11210,7 +11210,7 @@
         </is>
       </c>
       <c r="D17" s="115">
-        <f>IF(J19&lt;=0,"n.m.",I19/J19)</f>
+        <f>IF(I19&lt;=0,"n.m.",H19/I19)</f>
         <v/>
       </c>
       <c r="H17" s="116" t="n">
@@ -11237,7 +11237,7 @@
         </is>
       </c>
       <c r="D18" s="115">
-        <f>IF(J20&lt;=0,"n.m.",I20/J20)</f>
+        <f>IF(I20&lt;=0,"n.m.",H20/I20)</f>
         <v/>
       </c>
       <c r="H18" s="116" t="n">
@@ -11264,7 +11264,7 @@
         </is>
       </c>
       <c r="D19" s="115">
-        <f>IF(J21&lt;=0,"n.m.",I21/J21)</f>
+        <f>IF(I21&lt;=0,"n.m.",H21/I21)</f>
         <v/>
       </c>
       <c r="H19" s="116" t="n">
@@ -11291,7 +11291,7 @@
         </is>
       </c>
       <c r="D20" s="115">
-        <f>IF(J22&lt;=0,"n.m.",I22/J22)</f>
+        <f>IF(I22&lt;=0,"n.m.",H22/I22)</f>
         <v/>
       </c>
       <c r="H20" s="116" t="n">
@@ -11318,7 +11318,7 @@
         </is>
       </c>
       <c r="D21" s="115">
-        <f>IF(J23&lt;=0,"n.m.",I23/J23)</f>
+        <f>IF(I23&lt;=0,"n.m.",H23/I23)</f>
         <v/>
       </c>
       <c r="H21" s="116" t="n">
@@ -11345,7 +11345,7 @@
         </is>
       </c>
       <c r="D22" s="115">
-        <f>IF(J24&lt;=0,"n.m.",I24/J24)</f>
+        <f>IF(I24&lt;=0,"n.m.",H24/I24)</f>
         <v/>
       </c>
       <c r="H22" s="116" t="n">
@@ -11372,7 +11372,7 @@
         </is>
       </c>
       <c r="D23" s="115">
-        <f>IF(J25&lt;=0,"n.m.",I25/J25)</f>
+        <f>IF(I25&lt;=0,"n.m.",H25/I25)</f>
         <v/>
       </c>
       <c r="H23" s="116" t="n">
@@ -11399,7 +11399,7 @@
         </is>
       </c>
       <c r="D24" s="115">
-        <f>IF(J26&lt;=0,"n.m.",I26/J26)</f>
+        <f>IF(I26&lt;=0,"n.m.",H26/I26)</f>
         <v/>
       </c>
       <c r="H24" s="116" t="n">
@@ -11426,7 +11426,7 @@
         </is>
       </c>
       <c r="D25" s="115">
-        <f>IF(J27&lt;=0,"n.m.",I27/J27)</f>
+        <f>IF(I27&lt;=0,"n.m.",H27/I27)</f>
         <v/>
       </c>
       <c r="H25" s="116" t="n">
@@ -11453,7 +11453,7 @@
         </is>
       </c>
       <c r="D26" s="115">
-        <f>IF(J28&lt;=0,"n.m.",I28/J28)</f>
+        <f>IF(I28&lt;=0,"n.m.",H28/I28)</f>
         <v/>
       </c>
       <c r="H26" s="116" t="n">
@@ -11480,7 +11480,7 @@
         </is>
       </c>
       <c r="D27" s="115">
-        <f>IF(J29&lt;=0,"n.m.",I29/J29)</f>
+        <f>IF(I29&lt;=0,"n.m.",H29/I29)</f>
         <v/>
       </c>
       <c r="H27" s="116" t="n">
@@ -11516,7 +11516,7 @@
         </is>
       </c>
       <c r="D31" s="115">
-        <f>AVERAGE(E19,E22,E21,E23,E25,E27,E29)</f>
+        <f>AVERAGE(D19,D22,D21,D23,D25,D27,D29)</f>
         <v/>
       </c>
     </row>
@@ -11537,7 +11537,7 @@
         </is>
       </c>
       <c r="D32" s="115">
-        <f>AVERAGE(E19,E21,E22,E23,E24,E25,E26,E27,E28,E29)</f>
+        <f>AVERAGE(D19,D21,D22,D23,D24,D25,D26,D27,D28,D29)</f>
         <v/>
       </c>
     </row>
@@ -11585,7 +11585,7 @@
         </is>
       </c>
       <c r="D38" s="94">
-        <f>E45-E44</f>
+        <f>D45-D44</f>
         <v/>
       </c>
     </row>
@@ -11659,11 +11659,11 @@
         <v>8</v>
       </c>
       <c r="F42" s="121">
-        <f>(E6*E57+E8)/E9</f>
+        <f>(D6*D57+D8)/D9</f>
         <v/>
       </c>
       <c r="G42" s="121">
-        <f>(E6*F57+E8)/E9</f>
+        <f>(D6*E57+D8)/D9</f>
         <v/>
       </c>
     </row>
@@ -11688,7 +11688,7 @@
         <v/>
       </c>
       <c r="F43" s="122">
-        <f>(E6*E58+E8)/E9</f>
+        <f>(D6*D58+D8)/D9</f>
         <v/>
       </c>
     </row>
@@ -11717,11 +11717,11 @@
         <v>18</v>
       </c>
       <c r="F44" s="121">
-        <f>E7*E59</f>
+        <f>D7*D59</f>
         <v/>
       </c>
       <c r="G44" s="121">
-        <f>E7*F59</f>
+        <f>D7*E59</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix WACC empty numbers: bake col E values, guard value columns in merge
- Hardcode all 24 WACC col E cells from unaltered formulas so Excel shows
  numbers without recalc (E41 = 8.98%, rf 4.8%, ERP 6%, beta 0.84, CoE 9.86%)
- Add VALUE_COLS guard so Ctrl+F cleanup never clears col E or scenario matrices
- Audit confirms Scenarios/NOPAT/DCF value columns intact vs unaltered

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_final.xlsx
+++ b/LULU/model18_final.xlsx
@@ -1443,9 +1443,8 @@
         </is>
       </c>
       <c r="D10" s="19" t="n"/>
-      <c r="E10" s="25">
-        <f>E8*E9</f>
-        <v/>
+      <c r="E10" s="25" t="n">
+        <v>11138000</v>
       </c>
     </row>
     <row r="11" ht="28" customHeight="1">
@@ -1503,9 +1502,8 @@
           <t>Total debt equivalents</t>
         </is>
       </c>
-      <c r="E14" s="25">
-        <f>E11+E13</f>
-        <v/>
+      <c r="E14" s="25" t="n">
+        <v>1798441</v>
       </c>
     </row>
     <row r="15"/>
@@ -1596,9 +1594,8 @@
         </is>
       </c>
       <c r="D20" s="19" t="n"/>
-      <c r="E20" s="28">
-        <f>E18/E19</f>
-        <v/>
+      <c r="E20" s="28" t="n">
+        <v>0.1921005385996409</v>
       </c>
     </row>
     <row r="21" ht="28" customHeight="1">
@@ -1639,9 +1636,8 @@
         </is>
       </c>
       <c r="D22" s="19" t="n"/>
-      <c r="E22" s="28">
-        <f>E17/(1+(1-E5)*E20)</f>
-        <v/>
+      <c r="E22" s="28" t="n">
+        <v>0.7580629846494699</v>
       </c>
     </row>
     <row r="23" ht="28" customHeight="1">
@@ -1661,9 +1657,8 @@
         </is>
       </c>
       <c r="D23" s="19" t="n"/>
-      <c r="E23" s="28">
-        <f>E14/E10</f>
-        <v/>
+      <c r="E23" s="28" t="n">
+        <v>0.161468935176872</v>
       </c>
     </row>
     <row r="24" ht="28" customHeight="1">
@@ -1704,9 +1699,8 @@
         </is>
       </c>
       <c r="D25" s="19" t="n"/>
-      <c r="E25" s="29">
-        <f>E22*(1+(1-E5)*E23)</f>
-        <v/>
+      <c r="E25" s="29" t="n">
+        <v>0.8437455206993159</v>
       </c>
     </row>
     <row r="26">
@@ -1757,9 +1751,8 @@
           <t>Cost of equity = rf + β × ERP</t>
         </is>
       </c>
-      <c r="E32" s="30">
-        <f>E3+E25*E4</f>
-        <v/>
+      <c r="E32" s="30" t="n">
+        <v>0.09862473124195895</v>
       </c>
     </row>
     <row r="33"/>
@@ -1797,9 +1790,8 @@
           <t>After-tax cost of debt</t>
         </is>
       </c>
-      <c r="E36" s="31">
-        <f>E35*(1-E5)</f>
-        <v/>
+      <c r="E36" s="31" t="n">
+        <v>0.035</v>
       </c>
     </row>
     <row r="37"/>
@@ -1827,9 +1819,8 @@
         </is>
       </c>
       <c r="D39" s="19" t="n"/>
-      <c r="E39" s="32">
-        <f>E10/(E10+E14)</f>
-        <v/>
+      <c r="E39" s="32" t="n">
+        <v>0.8609786880332851</v>
       </c>
     </row>
     <row r="40" ht="28" customHeight="1">
@@ -1849,9 +1840,8 @@
         </is>
       </c>
       <c r="D40" s="19" t="n"/>
-      <c r="E40" s="32">
-        <f>E14/(E10+E14)</f>
-        <v/>
+      <c r="E40" s="32" t="n">
+        <v>0.1390213119667148</v>
       </c>
     </row>
     <row r="41">
@@ -1860,9 +1850,8 @@
           <t>WACC</t>
         </is>
       </c>
-      <c r="E41" s="33">
-        <f>E39*E32+E40*E36</f>
-        <v/>
+      <c r="E41" s="33" t="n">
+        <v>0.08977953763117218</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Restore Excel outline +/- controls on collapsible column and row groups
Enable showOutlineSymbols on all sheets and re-apply column B-D / I-L
and detail row grouping so Justification walls expand in desktop Excel.

Co-authored-by: cag56988 <cag56988@usc.edu>
</commit_message>
<xml_diff>
--- a/LULU/model18_final.xlsx
+++ b/LULU/model18_final.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cover" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="WACC" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Revenue Drivers" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOPAT Bridge" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DCF" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Comps" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Cover" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="WACC" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Scenarios" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Revenue Drivers" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="NOPAT Bridge" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="DCF" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Comps" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1115,14 +1115,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B25"/>
+  <dimension ref="B2:B25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -1130,7 +1129,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -1145,7 +1143,6 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
@@ -1153,7 +1150,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="B9" s="5" t="inlineStr">
         <is>
@@ -1182,7 +1178,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="B14" s="5" t="inlineStr">
         <is>
@@ -1212,7 +1207,6 @@
         </is>
       </c>
     </row>
-    <row r="18"/>
     <row r="19">
       <c r="B19" s="5" t="inlineStr">
         <is>
@@ -1248,7 +1242,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25">
       <c r="B25" s="11" t="inlineStr">
         <is>
@@ -1376,7 +1369,6 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="6"/>
     <row r="7">
       <c r="A7" s="14" t="inlineStr">
         <is>
@@ -1506,7 +1498,6 @@
         <v>1798441</v>
       </c>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
@@ -1755,7 +1746,6 @@
         <v>0.09862473124195895</v>
       </c>
     </row>
-    <row r="33"/>
     <row r="34">
       <c r="A34" s="14" t="inlineStr">
         <is>
@@ -1794,7 +1784,6 @@
         <v>0.035</v>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -2436,7 +2425,6 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="23"/>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
@@ -4439,7 +4427,6 @@
         <v/>
       </c>
     </row>
-    <row r="130"/>
     <row r="131">
       <c r="A131" s="23" t="inlineStr">
         <is>
@@ -4497,7 +4484,6 @@
         <v/>
       </c>
     </row>
-    <row r="134"/>
     <row r="135">
       <c r="A135" s="26" t="inlineStr">
         <is>
@@ -4505,7 +4491,6 @@
         </is>
       </c>
     </row>
-    <row r="136"/>
     <row r="137">
       <c r="A137" s="14" t="inlineStr">
         <is>
@@ -6370,7 +6355,6 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="52" t="inlineStr">
         <is>
@@ -6898,7 +6882,6 @@
       </c>
       <c r="L34" s="19" t="n"/>
     </row>
-    <row r="35"/>
     <row r="36">
       <c r="A36" s="52" t="inlineStr">
         <is>
@@ -7122,7 +7105,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="52" t="inlineStr">
         <is>
@@ -7506,7 +7488,6 @@
       </c>
       <c r="L51" s="19" t="n"/>
     </row>
-    <row r="52"/>
     <row r="53">
       <c r="A53" s="52" t="inlineStr">
         <is>
@@ -7897,7 +7878,6 @@
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
       <c r="A6" s="52" t="inlineStr">
         <is>
@@ -8128,7 +8108,6 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14"/>
     <row r="15" hidden="1" outlineLevel="1">
       <c r="A15" s="73" t="inlineStr">
         <is>
@@ -9044,7 +9023,6 @@
         <v/>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="73" t="inlineStr">
         <is>
@@ -9381,7 +9359,11 @@
 .</t>
         </is>
       </c>
-      <c r="D4" s="85" t="n"/>
+      <c r="D4" s="85" t="inlineStr">
+        <is>
+          <t>'Revenue Drivers'!A1</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
@@ -10527,7 +10509,6 @@
         <v/>
       </c>
     </row>
-    <row r="39"/>
     <row r="40">
       <c r="A40" s="15" t="inlineStr">
         <is>
@@ -10770,8 +10751,6 @@
         <v/>
       </c>
     </row>
-    <row r="60"/>
-    <row r="61"/>
     <row r="62">
       <c r="A62" s="93" t="inlineStr">
         <is>
@@ -10790,7 +10769,6 @@
         </is>
       </c>
     </row>
-    <row r="64"/>
     <row r="65">
       <c r="A65" s="16" t="inlineStr">
         <is>
@@ -10851,7 +10829,6 @@
         <v/>
       </c>
     </row>
-    <row r="67"/>
     <row r="68">
       <c r="A68" s="16" t="inlineStr">
         <is>
@@ -10936,7 +10913,6 @@
         <v/>
       </c>
     </row>
-    <row r="71"/>
     <row r="72">
       <c r="A72" s="16" t="inlineStr">
         <is>
@@ -11057,7 +11033,6 @@
         <v/>
       </c>
     </row>
-    <row r="76"/>
     <row r="77">
       <c r="A77" s="16" t="inlineStr">
         <is>
@@ -11118,7 +11093,6 @@
         <v/>
       </c>
     </row>
-    <row r="79"/>
     <row r="80">
       <c r="A80" s="93" t="inlineStr">
         <is>
@@ -11152,7 +11126,11 @@
         <f>E46</f>
         <v/>
       </c>
-      <c r="M82" s="95" t="n"/>
+      <c r="M82" s="95" t="inlineStr">
+        <is>
+          <t>'Comps'!A45</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="16" t="inlineStr">
@@ -11198,7 +11176,6 @@
         <v/>
       </c>
     </row>
-    <row r="87"/>
     <row r="88">
       <c r="A88" s="93" t="inlineStr">
         <is>
@@ -11305,8 +11282,6 @@
       </c>
       <c r="D94" s="26" t="n"/>
     </row>
-    <row r="95"/>
-    <row r="96"/>
     <row r="97">
       <c r="A97" s="93" t="inlineStr">
         <is>
@@ -11783,7 +11758,6 @@
         <v/>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
@@ -12158,7 +12132,6 @@
         <v>407521</v>
       </c>
     </row>
-    <row r="30"/>
     <row r="31">
       <c r="A31" s="14" t="inlineStr">
         <is>
@@ -12245,7 +12218,6 @@
         </is>
       </c>
     </row>
-    <row r="37"/>
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
@@ -12309,7 +12281,6 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
     <row r="43">
       <c r="A43" s="14" t="inlineStr">
         <is>
@@ -12399,7 +12370,6 @@
         </is>
       </c>
     </row>
-    <row r="54"/>
     <row r="55">
       <c r="A55" s="14" t="inlineStr">
         <is>
@@ -12564,7 +12534,6 @@
         <v/>
       </c>
     </row>
-    <row r="61"/>
     <row r="62" ht="28" customHeight="1">
       <c r="A62" s="124" t="inlineStr">
         <is>

</xml_diff>